<commit_message>
Fix full Gujarat supplier-wise stock to include all store and warehouse stock
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DwJnqVusC3tRSWnF3Qvwz
</commit_message>
<xml_diff>
--- a/docs/Supplier_wise_Full_GJ.xlsx
+++ b/docs/Supplier_wise_Full_GJ.xlsx
@@ -1370,13 +1370,13 @@
         <v>54255889</v>
       </c>
       <c r="P2" s="1">
-        <v>282991</v>
+        <v>303751</v>
       </c>
       <c r="Q2" s="1">
-        <v>23708597</v>
+        <v>25252505</v>
       </c>
       <c r="R2" s="2">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>145</v>
@@ -1429,13 +1429,13 @@
         <v>45524507</v>
       </c>
       <c r="P3" s="1">
-        <v>129700</v>
+        <v>136428</v>
       </c>
       <c r="Q3" s="1">
-        <v>23338272</v>
+        <v>24486238</v>
       </c>
       <c r="R3" s="2">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
       <c r="S3" s="1" t="s">
         <v>146</v>
@@ -1488,10 +1488,10 @@
         <v>20240180</v>
       </c>
       <c r="P4" s="1">
-        <v>12140</v>
+        <v>12837</v>
       </c>
       <c r="Q4" s="1">
-        <v>1137858</v>
+        <v>1223754</v>
       </c>
       <c r="R4" s="2">
         <v>0.2</v>
@@ -1547,10 +1547,10 @@
         <v>15679727</v>
       </c>
       <c r="P5" s="1">
-        <v>67373</v>
+        <v>68554</v>
       </c>
       <c r="Q5" s="1">
-        <v>2742626</v>
+        <v>2828335</v>
       </c>
       <c r="R5" s="2">
         <v>1.1</v>
@@ -1606,13 +1606,13 @@
         <v>14141465</v>
       </c>
       <c r="P6" s="1">
-        <v>21408</v>
+        <v>23610</v>
       </c>
       <c r="Q6" s="1">
-        <v>5847457</v>
+        <v>6500477</v>
       </c>
       <c r="R6" s="2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="S6" s="1" t="s">
         <v>149</v>
@@ -1665,10 +1665,10 @@
         <v>12011598</v>
       </c>
       <c r="P7" s="1">
-        <v>13679</v>
+        <v>14147</v>
       </c>
       <c r="Q7" s="1">
-        <v>3446164</v>
+        <v>3552844</v>
       </c>
       <c r="R7" s="2">
         <v>1.7</v>
@@ -1724,10 +1724,10 @@
         <v>9717919</v>
       </c>
       <c r="P8" s="1">
-        <v>42622</v>
+        <v>44641</v>
       </c>
       <c r="Q8" s="1">
-        <v>2339330</v>
+        <v>2528189</v>
       </c>
       <c r="R8" s="2">
         <v>1</v>
@@ -1783,10 +1783,10 @@
         <v>9534356</v>
       </c>
       <c r="P9" s="1">
-        <v>45592</v>
+        <v>47124</v>
       </c>
       <c r="Q9" s="1">
-        <v>1760405</v>
+        <v>1829193</v>
       </c>
       <c r="R9" s="2">
         <v>1.1</v>
@@ -1842,10 +1842,10 @@
         <v>9145683</v>
       </c>
       <c r="P10" s="1">
-        <v>64494</v>
+        <v>66050</v>
       </c>
       <c r="Q10" s="1">
-        <v>1867763</v>
+        <v>2043610</v>
       </c>
       <c r="R10" s="2">
         <v>1.2</v>
@@ -1901,13 +1901,13 @@
         <v>7717533</v>
       </c>
       <c r="P11" s="1">
-        <v>40663</v>
+        <v>42834</v>
       </c>
       <c r="Q11" s="1">
-        <v>3936910</v>
+        <v>4178415</v>
       </c>
       <c r="R11" s="2">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="S11" s="1" t="s">
         <v>154</v>
@@ -1960,13 +1960,13 @@
         <v>7582485</v>
       </c>
       <c r="P12" s="1">
-        <v>21256</v>
+        <v>22259</v>
       </c>
       <c r="Q12" s="1">
-        <v>3199031</v>
+        <v>3347660</v>
       </c>
       <c r="R12" s="2">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="S12" s="1" t="s">
         <v>155</v>
@@ -2019,10 +2019,10 @@
         <v>7324462</v>
       </c>
       <c r="P13" s="1">
-        <v>38832</v>
+        <v>39820</v>
       </c>
       <c r="Q13" s="1">
-        <v>2748271</v>
+        <v>2851192</v>
       </c>
       <c r="R13" s="2">
         <v>1.3</v>
@@ -2078,10 +2078,10 @@
         <v>5553389</v>
       </c>
       <c r="P14" s="1">
-        <v>33410</v>
+        <v>35058</v>
       </c>
       <c r="Q14" s="1">
-        <v>1255401</v>
+        <v>1330395</v>
       </c>
       <c r="R14" s="2">
         <v>1.3</v>
@@ -2137,13 +2137,13 @@
         <v>5479176</v>
       </c>
       <c r="P15" s="1">
-        <v>10991</v>
+        <v>11405</v>
       </c>
       <c r="Q15" s="1">
-        <v>1453998</v>
+        <v>1524618</v>
       </c>
       <c r="R15" s="2">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="S15" s="1" t="s">
         <v>158</v>
@@ -2196,10 +2196,10 @@
         <v>4805108</v>
       </c>
       <c r="P16" s="1">
-        <v>6605</v>
+        <v>7315</v>
       </c>
       <c r="Q16" s="1">
-        <v>802384</v>
+        <v>889693</v>
       </c>
       <c r="R16" s="2">
         <v>0.9</v>
@@ -2255,13 +2255,13 @@
         <v>4518071</v>
       </c>
       <c r="P17" s="1">
-        <v>9527</v>
+        <v>11325</v>
       </c>
       <c r="Q17" s="1">
-        <v>423606</v>
+        <v>511896</v>
       </c>
       <c r="R17" s="2">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="S17" s="1" t="s">
         <v>160</v>
@@ -2314,13 +2314,13 @@
         <v>4334035</v>
       </c>
       <c r="P18" s="1">
-        <v>6054</v>
+        <v>6425</v>
       </c>
       <c r="Q18" s="1">
-        <v>920395</v>
+        <v>964848</v>
       </c>
       <c r="R18" s="2">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="S18" s="1" t="s">
         <v>161</v>
@@ -2373,13 +2373,13 @@
         <v>4216981</v>
       </c>
       <c r="P19" s="1">
-        <v>5374</v>
+        <v>5763</v>
       </c>
       <c r="Q19" s="1">
-        <v>866785</v>
+        <v>926159</v>
       </c>
       <c r="R19" s="2">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="S19" s="1" t="s">
         <v>162</v>
@@ -2432,13 +2432,13 @@
         <v>3849754</v>
       </c>
       <c r="P20" s="1">
-        <v>4955</v>
+        <v>5384</v>
       </c>
       <c r="Q20" s="1">
-        <v>552635</v>
+        <v>604160</v>
       </c>
       <c r="R20" s="2">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="S20" s="1" t="s">
         <v>163</v>
@@ -2491,13 +2491,13 @@
         <v>3564517</v>
       </c>
       <c r="P21" s="1">
-        <v>9202</v>
+        <v>9639</v>
       </c>
       <c r="Q21" s="1">
-        <v>1361837</v>
+        <v>1440432</v>
       </c>
       <c r="R21" s="2">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="S21" s="1" t="s">
         <v>164</v>
@@ -2550,10 +2550,10 @@
         <v>3485757</v>
       </c>
       <c r="P22" s="1">
-        <v>11994</v>
+        <v>12425</v>
       </c>
       <c r="Q22" s="1">
-        <v>743892</v>
+        <v>774102</v>
       </c>
       <c r="R22" s="2">
         <v>1.3</v>
@@ -2609,13 +2609,13 @@
         <v>3421998</v>
       </c>
       <c r="P23" s="1">
-        <v>5194</v>
+        <v>6098</v>
       </c>
       <c r="Q23" s="1">
-        <v>697620</v>
+        <v>768804</v>
       </c>
       <c r="R23" s="2">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="S23" s="1" t="s">
         <v>166</v>
@@ -2668,13 +2668,13 @@
         <v>3403556</v>
       </c>
       <c r="P24" s="1">
-        <v>14297</v>
+        <v>14861</v>
       </c>
       <c r="Q24" s="1">
-        <v>872174</v>
+        <v>900883</v>
       </c>
       <c r="R24" s="2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="S24" s="1" t="s">
         <v>167</v>
@@ -2727,13 +2727,13 @@
         <v>3153302</v>
       </c>
       <c r="P25" s="1">
-        <v>2552</v>
+        <v>2730</v>
       </c>
       <c r="Q25" s="1">
-        <v>479332</v>
+        <v>509718</v>
       </c>
       <c r="R25" s="2">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="S25" s="1" t="s">
         <v>168</v>
@@ -2786,13 +2786,13 @@
         <v>2901328</v>
       </c>
       <c r="P26" s="1">
-        <v>10910</v>
+        <v>11285</v>
       </c>
       <c r="Q26" s="1">
-        <v>985591</v>
+        <v>1029298</v>
       </c>
       <c r="R26" s="2">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="S26" s="1" t="s">
         <v>169</v>
@@ -2845,10 +2845,10 @@
         <v>2481407</v>
       </c>
       <c r="P27" s="1">
-        <v>6904</v>
+        <v>7086</v>
       </c>
       <c r="Q27" s="1">
-        <v>641183</v>
+        <v>658468</v>
       </c>
       <c r="R27" s="2">
         <v>1.5</v>
@@ -2904,13 +2904,13 @@
         <v>2373975</v>
       </c>
       <c r="P28" s="1">
-        <v>5461</v>
+        <v>6009</v>
       </c>
       <c r="Q28" s="1">
-        <v>433023</v>
+        <v>495653</v>
       </c>
       <c r="R28" s="2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="S28" s="1" t="s">
         <v>171</v>
@@ -2963,13 +2963,13 @@
         <v>2127393</v>
       </c>
       <c r="P29" s="1">
-        <v>5439</v>
+        <v>5943</v>
       </c>
       <c r="Q29" s="1">
-        <v>408169</v>
+        <v>459278</v>
       </c>
       <c r="R29" s="2">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="S29" s="1" t="s">
         <v>172</v>
@@ -3022,13 +3022,13 @@
         <v>2051386</v>
       </c>
       <c r="P30" s="1">
-        <v>5479</v>
+        <v>5862</v>
       </c>
       <c r="Q30" s="1">
-        <v>581868</v>
+        <v>633268</v>
       </c>
       <c r="R30" s="2">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="S30" s="1" t="s">
         <v>173</v>
@@ -3081,10 +3081,10 @@
         <v>1996475</v>
       </c>
       <c r="P31" s="1">
-        <v>3311</v>
+        <v>3224</v>
       </c>
       <c r="Q31" s="1">
-        <v>536163</v>
+        <v>537945</v>
       </c>
       <c r="R31" s="2">
         <v>1.6</v>
@@ -3140,13 +3140,13 @@
         <v>1992220</v>
       </c>
       <c r="P32" s="1">
-        <v>3699</v>
+        <v>4013</v>
       </c>
       <c r="Q32" s="1">
-        <v>601826</v>
+        <v>637402</v>
       </c>
       <c r="R32" s="2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="S32" s="1" t="s">
         <v>175</v>
@@ -3199,13 +3199,13 @@
         <v>1952923</v>
       </c>
       <c r="P33" s="1">
-        <v>1607</v>
+        <v>2225</v>
       </c>
       <c r="Q33" s="1">
-        <v>185280</v>
+        <v>252307</v>
       </c>
       <c r="R33" s="2">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="S33" s="1" t="s">
         <v>176</v>
@@ -3258,13 +3258,13 @@
         <v>1830717</v>
       </c>
       <c r="P34" s="1">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="Q34" s="1">
-        <v>34284</v>
+        <v>38277</v>
       </c>
       <c r="R34" s="2">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="S34" s="1" t="s">
         <v>177</v>
@@ -3317,13 +3317,13 @@
         <v>1729934</v>
       </c>
       <c r="P35" s="1">
-        <v>4880</v>
+        <v>4959</v>
       </c>
       <c r="Q35" s="1">
-        <v>956119</v>
+        <v>985941</v>
       </c>
       <c r="R35" s="2">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="S35" s="1" t="s">
         <v>178</v>
@@ -3376,10 +3376,10 @@
         <v>1719805</v>
       </c>
       <c r="P36" s="1">
-        <v>10208</v>
+        <v>10934</v>
       </c>
       <c r="Q36" s="1">
-        <v>283499</v>
+        <v>323928</v>
       </c>
       <c r="R36" s="2">
         <v>0.8</v>
@@ -3435,13 +3435,13 @@
         <v>1717791</v>
       </c>
       <c r="P37" s="1">
-        <v>6740</v>
+        <v>8101</v>
       </c>
       <c r="Q37" s="1">
-        <v>175784</v>
+        <v>205375</v>
       </c>
       <c r="R37" s="2">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="S37" s="1" t="s">
         <v>54</v>
@@ -3494,13 +3494,13 @@
         <v>1633719</v>
       </c>
       <c r="P38" s="1">
-        <v>6928</v>
+        <v>7279</v>
       </c>
       <c r="Q38" s="1">
-        <v>318090</v>
+        <v>332080</v>
       </c>
       <c r="R38" s="2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="S38" s="1" t="s">
         <v>179</v>
@@ -3553,10 +3553,10 @@
         <v>1613859</v>
       </c>
       <c r="P39" s="1">
-        <v>6000</v>
+        <v>6022</v>
       </c>
       <c r="Q39" s="1">
-        <v>743384</v>
+        <v>746454</v>
       </c>
       <c r="R39" s="2">
         <v>2.4</v>
@@ -3612,13 +3612,13 @@
         <v>1548859</v>
       </c>
       <c r="P40" s="1">
-        <v>1438</v>
+        <v>1620</v>
       </c>
       <c r="Q40" s="1">
-        <v>374317</v>
+        <v>424966</v>
       </c>
       <c r="R40" s="2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="S40" s="1" t="s">
         <v>57</v>
@@ -3671,13 +3671,13 @@
         <v>1536754</v>
       </c>
       <c r="P41" s="1">
-        <v>1395</v>
+        <v>1647</v>
       </c>
       <c r="Q41" s="1">
-        <v>411284</v>
+        <v>491474</v>
       </c>
       <c r="R41" s="2">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="S41" s="1" t="s">
         <v>181</v>
@@ -3730,13 +3730,13 @@
         <v>1502872</v>
       </c>
       <c r="P42" s="1">
-        <v>1084</v>
+        <v>1217</v>
       </c>
       <c r="Q42" s="1">
-        <v>209801</v>
+        <v>246815</v>
       </c>
       <c r="R42" s="2">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="S42" s="1" t="s">
         <v>182</v>
@@ -3789,10 +3789,10 @@
         <v>1414849</v>
       </c>
       <c r="P43" s="1">
-        <v>9391</v>
+        <v>9920</v>
       </c>
       <c r="Q43" s="1">
-        <v>275777</v>
+        <v>309308</v>
       </c>
       <c r="R43" s="2">
         <v>0.8</v>
@@ -3848,13 +3848,13 @@
         <v>1365547</v>
       </c>
       <c r="P44" s="1">
-        <v>2932</v>
+        <v>3112</v>
       </c>
       <c r="Q44" s="1">
-        <v>658564</v>
+        <v>706473</v>
       </c>
       <c r="R44" s="2">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="S44" s="1" t="s">
         <v>184</v>
@@ -3907,10 +3907,10 @@
         <v>1258947</v>
       </c>
       <c r="P45" s="1">
-        <v>11860</v>
+        <v>12000</v>
       </c>
       <c r="Q45" s="1">
-        <v>368280</v>
+        <v>374813</v>
       </c>
       <c r="R45" s="2">
         <v>1.6</v>
@@ -3966,13 +3966,13 @@
         <v>1222686</v>
       </c>
       <c r="P46" s="1">
-        <v>4836</v>
+        <v>5134</v>
       </c>
       <c r="Q46" s="1">
-        <v>211227</v>
+        <v>224587</v>
       </c>
       <c r="R46" s="2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="S46" s="1" t="s">
         <v>186</v>
@@ -4025,13 +4025,13 @@
         <v>1200781</v>
       </c>
       <c r="P47" s="1">
-        <v>9660</v>
+        <v>11440</v>
       </c>
       <c r="Q47" s="1">
-        <v>323964</v>
+        <v>366010</v>
       </c>
       <c r="R47" s="2">
-        <v>1.7</v>
+        <v>2</v>
       </c>
       <c r="S47" s="1" t="s">
         <v>187</v>
@@ -4084,10 +4084,10 @@
         <v>1168782</v>
       </c>
       <c r="P48" s="1">
-        <v>4165</v>
+        <v>4195</v>
       </c>
       <c r="Q48" s="1">
-        <v>425752</v>
+        <v>429023</v>
       </c>
       <c r="R48" s="2">
         <v>2</v>
@@ -4202,10 +4202,10 @@
         <v>1053912</v>
       </c>
       <c r="P50" s="1">
-        <v>2537</v>
+        <v>2556</v>
       </c>
       <c r="Q50" s="1">
-        <v>296371</v>
+        <v>297945</v>
       </c>
       <c r="R50" s="2">
         <v>1.4</v>
@@ -4261,10 +4261,10 @@
         <v>1050243</v>
       </c>
       <c r="P51" s="1">
-        <v>1275</v>
+        <v>1328</v>
       </c>
       <c r="Q51" s="1">
-        <v>431675</v>
+        <v>451461</v>
       </c>
       <c r="R51" s="2">
         <v>0.8</v>
@@ -4320,13 +4320,13 @@
         <v>962277</v>
       </c>
       <c r="P52" s="1">
-        <v>6065</v>
+        <v>6250</v>
       </c>
       <c r="Q52" s="1">
-        <v>687010</v>
+        <v>719335</v>
       </c>
       <c r="R52" s="2">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="S52" s="1" t="s">
         <v>192</v>
@@ -4379,13 +4379,13 @@
         <v>938957</v>
       </c>
       <c r="P53" s="1">
-        <v>1761</v>
+        <v>2116</v>
       </c>
       <c r="Q53" s="1">
-        <v>75983</v>
+        <v>102159</v>
       </c>
       <c r="R53" s="2">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="S53" s="1" t="s">
         <v>193</v>
@@ -4438,10 +4438,10 @@
         <v>917414</v>
       </c>
       <c r="P54" s="1">
-        <v>1221</v>
+        <v>1237</v>
       </c>
       <c r="Q54" s="1">
-        <v>180051</v>
+        <v>182947</v>
       </c>
       <c r="R54" s="2">
         <v>1.1</v>
@@ -4497,13 +4497,13 @@
         <v>869605</v>
       </c>
       <c r="P55" s="1">
-        <v>1050</v>
+        <v>1201</v>
       </c>
       <c r="Q55" s="1">
-        <v>314412</v>
+        <v>364427</v>
       </c>
       <c r="R55" s="2">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="S55" s="1" t="s">
         <v>195</v>
@@ -4556,13 +4556,13 @@
         <v>865930</v>
       </c>
       <c r="P56" s="1">
-        <v>1500</v>
+        <v>1542</v>
       </c>
       <c r="Q56" s="1">
-        <v>318152</v>
+        <v>332104</v>
       </c>
       <c r="R56" s="2">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="S56" s="1" t="s">
         <v>196</v>
@@ -4615,10 +4615,10 @@
         <v>795798</v>
       </c>
       <c r="P57" s="1">
-        <v>889</v>
+        <v>880</v>
       </c>
       <c r="Q57" s="1">
-        <v>300454</v>
+        <v>302103</v>
       </c>
       <c r="R57" s="2">
         <v>1.6</v>
@@ -4674,10 +4674,10 @@
         <v>725876</v>
       </c>
       <c r="P58" s="1">
-        <v>9399</v>
+        <v>9538</v>
       </c>
       <c r="Q58" s="1">
-        <v>499040</v>
+        <v>505640</v>
       </c>
       <c r="R58" s="2">
         <v>4.2</v>
@@ -4733,13 +4733,13 @@
         <v>705719</v>
       </c>
       <c r="P59" s="1">
-        <v>4839</v>
+        <v>5139</v>
       </c>
       <c r="Q59" s="1">
-        <v>342558</v>
+        <v>365301</v>
       </c>
       <c r="R59" s="2">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="S59" s="1" t="s">
         <v>199</v>
@@ -4792,10 +4792,10 @@
         <v>698835</v>
       </c>
       <c r="P60" s="1">
-        <v>1881</v>
+        <v>1902</v>
       </c>
       <c r="Q60" s="1">
-        <v>150430</v>
+        <v>151898</v>
       </c>
       <c r="R60" s="2">
         <v>1.3</v>
@@ -4851,13 +4851,13 @@
         <v>587724</v>
       </c>
       <c r="P61" s="1">
-        <v>2863</v>
+        <v>4372</v>
       </c>
       <c r="Q61" s="1">
-        <v>81353</v>
+        <v>114338</v>
       </c>
       <c r="R61" s="2">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="S61" s="1" t="s">
         <v>201</v>
@@ -4969,10 +4969,10 @@
         <v>576776</v>
       </c>
       <c r="P63" s="1">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="Q63" s="1">
-        <v>104280</v>
+        <v>105850</v>
       </c>
       <c r="R63" s="2">
         <v>1.2</v>
@@ -5028,13 +5028,13 @@
         <v>569994</v>
       </c>
       <c r="P64" s="1">
-        <v>1126</v>
+        <v>1187</v>
       </c>
       <c r="Q64" s="1">
-        <v>279014</v>
+        <v>284460</v>
       </c>
       <c r="R64" s="2">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
       <c r="S64" s="1" t="s">
         <v>203</v>
@@ -5087,13 +5087,13 @@
         <v>543885</v>
       </c>
       <c r="P65" s="1">
-        <v>574</v>
+        <v>606</v>
       </c>
       <c r="Q65" s="1">
-        <v>93006</v>
+        <v>100035</v>
       </c>
       <c r="R65" s="2">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="S65" s="1" t="s">
         <v>204</v>
@@ -5146,13 +5146,13 @@
         <v>525089</v>
       </c>
       <c r="P66" s="1">
-        <v>807</v>
+        <v>823</v>
       </c>
       <c r="Q66" s="1">
-        <v>160586</v>
+        <v>170585</v>
       </c>
       <c r="R66" s="2">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="S66" s="1" t="s">
         <v>205</v>
@@ -5205,13 +5205,13 @@
         <v>506044</v>
       </c>
       <c r="P67" s="1">
-        <v>17344</v>
+        <v>17552</v>
       </c>
       <c r="Q67" s="1">
-        <v>845962</v>
+        <v>847060</v>
       </c>
       <c r="R67" s="2">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="S67" s="1" t="s">
         <v>206</v>
@@ -5264,13 +5264,13 @@
         <v>503475</v>
       </c>
       <c r="P68" s="1">
-        <v>3691</v>
+        <v>4729</v>
       </c>
       <c r="Q68" s="1">
-        <v>424583</v>
+        <v>590344</v>
       </c>
       <c r="R68" s="2">
-        <v>4</v>
+        <v>5.1</v>
       </c>
       <c r="S68" s="1" t="s">
         <v>207</v>
@@ -5323,10 +5323,10 @@
         <v>494215</v>
       </c>
       <c r="P69" s="1">
-        <v>2182</v>
+        <v>2169</v>
       </c>
       <c r="Q69" s="1">
-        <v>60487</v>
+        <v>82913</v>
       </c>
       <c r="R69" s="2">
         <v>0.7</v>
@@ -5382,13 +5382,13 @@
         <v>481799</v>
       </c>
       <c r="P70" s="1">
-        <v>1927</v>
+        <v>2087</v>
       </c>
       <c r="Q70" s="1">
-        <v>126025</v>
+        <v>135680</v>
       </c>
       <c r="R70" s="2">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="S70" s="1" t="s">
         <v>208</v>
@@ -5441,13 +5441,13 @@
         <v>446545</v>
       </c>
       <c r="P71" s="1">
-        <v>2379</v>
+        <v>2700</v>
       </c>
       <c r="Q71" s="1">
-        <v>204901</v>
+        <v>228614</v>
       </c>
       <c r="R71" s="2">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="S71" s="1" t="s">
         <v>209</v>
@@ -5500,13 +5500,13 @@
         <v>443725</v>
       </c>
       <c r="P72" s="1">
-        <v>866</v>
+        <v>926</v>
       </c>
       <c r="Q72" s="1">
-        <v>80986</v>
+        <v>84293</v>
       </c>
       <c r="R72" s="2">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="S72" s="1" t="s">
         <v>210</v>
@@ -5559,10 +5559,10 @@
         <v>419678</v>
       </c>
       <c r="P73" s="1">
-        <v>3280</v>
+        <v>3336</v>
       </c>
       <c r="Q73" s="1">
-        <v>315608</v>
+        <v>328466</v>
       </c>
       <c r="R73" s="2">
         <v>2.2</v>
@@ -5618,13 +5618,13 @@
         <v>416146</v>
       </c>
       <c r="P74" s="1">
-        <v>526</v>
+        <v>552</v>
       </c>
       <c r="Q74" s="1">
-        <v>321039</v>
+        <v>325689</v>
       </c>
       <c r="R74" s="2">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="S74" s="1" t="s">
         <v>212</v>
@@ -5677,13 +5677,13 @@
         <v>399232</v>
       </c>
       <c r="P75" s="1">
-        <v>3386</v>
+        <v>3056</v>
       </c>
       <c r="Q75" s="1">
-        <v>145090</v>
+        <v>145900</v>
       </c>
       <c r="R75" s="2">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="S75" s="1" t="s">
         <v>213</v>
@@ -5736,13 +5736,13 @@
         <v>371222</v>
       </c>
       <c r="P76" s="1">
-        <v>3480</v>
+        <v>3560</v>
       </c>
       <c r="Q76" s="1">
-        <v>533698</v>
+        <v>542018</v>
       </c>
       <c r="R76" s="2">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
       <c r="S76" s="1" t="s">
         <v>214</v>
@@ -5795,13 +5795,13 @@
         <v>367850</v>
       </c>
       <c r="P77" s="1">
-        <v>1591</v>
+        <v>1618</v>
       </c>
       <c r="Q77" s="1">
-        <v>142194</v>
+        <v>147283</v>
       </c>
       <c r="R77" s="2">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
       <c r="S77" s="1" t="s">
         <v>215</v>
@@ -5854,13 +5854,13 @@
         <v>363780</v>
       </c>
       <c r="P78" s="1">
-        <v>3243</v>
+        <v>3293</v>
       </c>
       <c r="Q78" s="1">
-        <v>360614</v>
+        <v>365008</v>
       </c>
       <c r="R78" s="2">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="S78" s="1" t="s">
         <v>216</v>
@@ -5913,10 +5913,10 @@
         <v>356405</v>
       </c>
       <c r="P79" s="1">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="Q79" s="1">
-        <v>85098</v>
+        <v>85170</v>
       </c>
       <c r="R79" s="2">
         <v>1.5</v>
@@ -5972,10 +5972,10 @@
         <v>353335</v>
       </c>
       <c r="P80" s="1">
-        <v>1586</v>
+        <v>1598</v>
       </c>
       <c r="Q80" s="1">
-        <v>164614</v>
+        <v>165988</v>
       </c>
       <c r="R80" s="2">
         <v>2.7</v>
@@ -6031,13 +6031,13 @@
         <v>335048</v>
       </c>
       <c r="P81" s="1">
-        <v>1589</v>
+        <v>1717</v>
       </c>
       <c r="Q81" s="1">
-        <v>143454</v>
+        <v>155882</v>
       </c>
       <c r="R81" s="2">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="S81" s="1" t="s">
         <v>219</v>
@@ -6090,10 +6090,10 @@
         <v>312069</v>
       </c>
       <c r="P82" s="1">
-        <v>1805</v>
+        <v>1887</v>
       </c>
       <c r="Q82" s="1">
-        <v>112586</v>
+        <v>115063</v>
       </c>
       <c r="R82" s="2">
         <v>1</v>
@@ -6149,10 +6149,10 @@
         <v>306511</v>
       </c>
       <c r="P83" s="1">
-        <v>852</v>
+        <v>887</v>
       </c>
       <c r="Q83" s="1">
-        <v>77956</v>
+        <v>82365</v>
       </c>
       <c r="R83" s="2">
         <v>1.2</v>
@@ -6208,13 +6208,13 @@
         <v>306374</v>
       </c>
       <c r="P84" s="1">
-        <v>927</v>
+        <v>956</v>
       </c>
       <c r="Q84" s="1">
-        <v>92476</v>
+        <v>95158</v>
       </c>
       <c r="R84" s="2">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="S84" s="1" t="s">
         <v>222</v>
@@ -6267,10 +6267,10 @@
         <v>303328</v>
       </c>
       <c r="P85" s="1">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="Q85" s="1">
-        <v>6000</v>
+        <v>6152</v>
       </c>
       <c r="R85" s="2">
         <v>0.1</v>
@@ -6326,7 +6326,7 @@
         <v>287372</v>
       </c>
       <c r="P86" s="1">
-        <v>1324</v>
+        <v>1314</v>
       </c>
       <c r="Q86" s="1">
         <v>182207</v>
@@ -6385,13 +6385,13 @@
         <v>258797</v>
       </c>
       <c r="P87" s="1">
-        <v>751</v>
+        <v>871</v>
       </c>
       <c r="Q87" s="1">
-        <v>53938</v>
+        <v>62770</v>
       </c>
       <c r="R87" s="2">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
       <c r="S87" s="1" t="s">
         <v>225</v>
@@ -6444,13 +6444,13 @@
         <v>257112</v>
       </c>
       <c r="P88" s="1">
-        <v>374</v>
+        <v>623</v>
       </c>
       <c r="Q88" s="1">
-        <v>69212</v>
+        <v>98854</v>
       </c>
       <c r="R88" s="2">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="S88" s="1" t="s">
         <v>226</v>
@@ -6503,10 +6503,10 @@
         <v>247853</v>
       </c>
       <c r="P89" s="1">
-        <v>5678</v>
+        <v>5680</v>
       </c>
       <c r="Q89" s="1">
-        <v>824852</v>
+        <v>824972</v>
       </c>
       <c r="R89" s="2">
         <v>11.4</v>
@@ -6562,13 +6562,13 @@
         <v>247507</v>
       </c>
       <c r="P90" s="1">
-        <v>610</v>
+        <v>603</v>
       </c>
       <c r="Q90" s="1">
-        <v>101210</v>
+        <v>102296</v>
       </c>
       <c r="R90" s="2">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="S90" s="1" t="s">
         <v>228</v>
@@ -6621,13 +6621,13 @@
         <v>232232</v>
       </c>
       <c r="P91" s="1">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="Q91" s="1">
-        <v>9155</v>
+        <v>18737</v>
       </c>
       <c r="R91" s="2">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="S91" s="1" t="s">
         <v>229</v>
@@ -6680,13 +6680,13 @@
         <v>228869</v>
       </c>
       <c r="P92" s="1">
-        <v>834</v>
+        <v>959</v>
       </c>
       <c r="Q92" s="1">
-        <v>53338</v>
+        <v>61533</v>
       </c>
       <c r="R92" s="2">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="S92" s="1" t="s">
         <v>230</v>
@@ -6739,13 +6739,13 @@
         <v>222516</v>
       </c>
       <c r="P93" s="1">
-        <v>4748</v>
+        <v>4873</v>
       </c>
       <c r="Q93" s="1">
-        <v>565737</v>
+        <v>582922</v>
       </c>
       <c r="R93" s="2">
-        <v>11.7</v>
+        <v>12</v>
       </c>
       <c r="S93" s="1" t="s">
         <v>231</v>
@@ -6798,10 +6798,10 @@
         <v>209820</v>
       </c>
       <c r="P94" s="1">
-        <v>3478</v>
+        <v>3500</v>
       </c>
       <c r="Q94" s="1">
-        <v>188378</v>
+        <v>189934</v>
       </c>
       <c r="R94" s="2">
         <v>5.7</v>
@@ -6857,10 +6857,10 @@
         <v>205272</v>
       </c>
       <c r="P95" s="1">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="Q95" s="1">
-        <v>122694</v>
+        <v>123683</v>
       </c>
       <c r="R95" s="2">
         <v>2.7</v>
@@ -6916,10 +6916,10 @@
         <v>188616</v>
       </c>
       <c r="P96" s="1">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="Q96" s="1">
-        <v>58343</v>
+        <v>58593</v>
       </c>
       <c r="R96" s="2">
         <v>1.8</v>
@@ -6975,13 +6975,13 @@
         <v>181446</v>
       </c>
       <c r="P97" s="1">
-        <v>1773</v>
+        <v>1816</v>
       </c>
       <c r="Q97" s="1">
-        <v>112606</v>
+        <v>117499</v>
       </c>
       <c r="R97" s="2">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="S97" s="1" t="s">
         <v>235</v>
@@ -7093,13 +7093,13 @@
         <v>166081</v>
       </c>
       <c r="P99" s="1">
-        <v>1276</v>
+        <v>1304</v>
       </c>
       <c r="Q99" s="1">
-        <v>111764</v>
+        <v>116369</v>
       </c>
       <c r="R99" s="2">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="S99" s="1" t="s">
         <v>237</v>
@@ -7152,10 +7152,10 @@
         <v>165708</v>
       </c>
       <c r="P100" s="1">
-        <v>505</v>
+        <v>526</v>
       </c>
       <c r="Q100" s="1">
-        <v>25766</v>
+        <v>26563</v>
       </c>
       <c r="R100" s="2">
         <v>0.9</v>
@@ -7211,13 +7211,13 @@
         <v>162658</v>
       </c>
       <c r="P101" s="1">
-        <v>2464</v>
+        <v>2785</v>
       </c>
       <c r="Q101" s="1">
-        <v>78163</v>
+        <v>84261</v>
       </c>
       <c r="R101" s="2">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="S101" s="1" t="s">
         <v>239</v>
@@ -7270,10 +7270,10 @@
         <v>160758</v>
       </c>
       <c r="P102" s="1">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="Q102" s="1">
-        <v>119198</v>
+        <v>119460</v>
       </c>
       <c r="R102" s="2">
         <v>4.4</v>
@@ -7329,13 +7329,13 @@
         <v>155919</v>
       </c>
       <c r="P103" s="1">
-        <v>1234</v>
+        <v>1332</v>
       </c>
       <c r="Q103" s="1">
-        <v>52432</v>
+        <v>56555</v>
       </c>
       <c r="R103" s="2">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="S103" s="1" t="s">
         <v>241</v>
@@ -7388,10 +7388,10 @@
         <v>145054</v>
       </c>
       <c r="P104" s="1">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="Q104" s="1">
-        <v>118606</v>
+        <v>120437</v>
       </c>
       <c r="R104" s="2">
         <v>3.3</v>
@@ -7447,10 +7447,10 @@
         <v>125380</v>
       </c>
       <c r="P105" s="1">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="Q105" s="1">
-        <v>36241</v>
+        <v>37981</v>
       </c>
       <c r="R105" s="2">
         <v>1.7</v>
@@ -7506,10 +7506,10 @@
         <v>119439</v>
       </c>
       <c r="P106" s="1">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="Q106" s="1">
-        <v>36775</v>
+        <v>36824</v>
       </c>
       <c r="R106" s="2">
         <v>1.8</v>
@@ -7624,13 +7624,13 @@
         <v>108899</v>
       </c>
       <c r="P108" s="1">
-        <v>416</v>
+        <v>462</v>
       </c>
       <c r="Q108" s="1">
-        <v>21236</v>
+        <v>23593</v>
       </c>
       <c r="R108" s="2">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="S108" s="1" t="s">
         <v>246</v>
@@ -7683,13 +7683,13 @@
         <v>85756</v>
       </c>
       <c r="P109" s="1">
-        <v>79</v>
+        <v>192</v>
       </c>
       <c r="Q109" s="1">
-        <v>5286</v>
+        <v>17455</v>
       </c>
       <c r="R109" s="2">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="S109" s="1" t="s">
         <v>247</v>
@@ -7742,10 +7742,10 @@
         <v>77595</v>
       </c>
       <c r="P110" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q110" s="1">
-        <v>258</v>
+        <v>295</v>
       </c>
       <c r="R110" s="2">
         <v>0</v>
@@ -7860,10 +7860,10 @@
         <v>70476</v>
       </c>
       <c r="P112" s="1">
-        <v>422</v>
+        <v>442</v>
       </c>
       <c r="Q112" s="1">
-        <v>13014</v>
+        <v>13614</v>
       </c>
       <c r="R112" s="2">
         <v>1.1</v>
@@ -7919,13 +7919,13 @@
         <v>65173</v>
       </c>
       <c r="P113" s="1">
-        <v>261</v>
+        <v>387</v>
       </c>
       <c r="Q113" s="1">
-        <v>19109</v>
+        <v>26053</v>
       </c>
       <c r="R113" s="2">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="S113" s="1" t="s">
         <v>251</v>
@@ -7978,13 +7978,13 @@
         <v>61440</v>
       </c>
       <c r="P114" s="1">
-        <v>166</v>
+        <v>258</v>
       </c>
       <c r="Q114" s="1">
-        <v>7950</v>
+        <v>10610</v>
       </c>
       <c r="R114" s="2">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="S114" s="1" t="s">
         <v>252</v>
@@ -8155,13 +8155,13 @@
         <v>36954</v>
       </c>
       <c r="P117" s="1">
-        <v>2186</v>
+        <v>2263</v>
       </c>
       <c r="Q117" s="1">
-        <v>64866</v>
+        <v>67176</v>
       </c>
       <c r="R117" s="2">
-        <v>10.6</v>
+        <v>11</v>
       </c>
       <c r="S117" s="1" t="s">
         <v>255</v>
@@ -8214,13 +8214,13 @@
         <v>34286</v>
       </c>
       <c r="P118" s="1">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="Q118" s="1">
-        <v>33271</v>
+        <v>33886</v>
       </c>
       <c r="R118" s="2">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
       <c r="S118" s="1" t="s">
         <v>256</v>
@@ -8273,10 +8273,10 @@
         <v>30897</v>
       </c>
       <c r="P119" s="1">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="Q119" s="1">
-        <v>10353</v>
+        <v>10473</v>
       </c>
       <c r="R119" s="2">
         <v>0</v>
@@ -8332,10 +8332,10 @@
         <v>25268</v>
       </c>
       <c r="P120" s="1">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Q120" s="1">
-        <v>9791</v>
+        <v>9855</v>
       </c>
       <c r="R120" s="2">
         <v>2.5</v>
@@ -8450,13 +8450,13 @@
         <v>2439</v>
       </c>
       <c r="P122" s="1">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="Q122" s="1">
-        <v>1347</v>
+        <v>2089</v>
       </c>
       <c r="R122" s="2">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
       <c r="S122" s="1" t="s">
         <v>260</v>
@@ -8568,13 +8568,13 @@
         <v>94</v>
       </c>
       <c r="P124" s="1">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q124" s="1">
-        <v>1030</v>
+        <v>1201</v>
       </c>
       <c r="R124" s="2">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="S124" s="1" t="s">
         <v>262</v>
@@ -8627,10 +8627,10 @@
         <v>0</v>
       </c>
       <c r="P125" s="1">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="Q125" s="1">
-        <v>1102</v>
+        <v>1159</v>
       </c>
       <c r="S125" s="1" t="s">
         <v>263</v>
@@ -8683,10 +8683,10 @@
         <v>0</v>
       </c>
       <c r="P126" s="1">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q126" s="1">
-        <v>40</v>
+        <v>556</v>
       </c>
       <c r="S126" s="1" t="s">
         <v>264</v>
@@ -8882,13 +8882,13 @@
         <v>54255889</v>
       </c>
       <c r="Q2" s="1">
-        <v>282991</v>
+        <v>303751</v>
       </c>
       <c r="R2" s="1">
-        <v>23708597</v>
+        <v>25252505</v>
       </c>
       <c r="S2" s="2">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -8941,13 +8941,13 @@
         <v>45524507</v>
       </c>
       <c r="Q3" s="1">
-        <v>129700</v>
+        <v>136428</v>
       </c>
       <c r="R3" s="1">
-        <v>23338272</v>
+        <v>24486238</v>
       </c>
       <c r="S3" s="2">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -9000,10 +9000,10 @@
         <v>20240180</v>
       </c>
       <c r="Q4" s="1">
-        <v>12140</v>
+        <v>12837</v>
       </c>
       <c r="R4" s="1">
-        <v>1137858</v>
+        <v>1223754</v>
       </c>
       <c r="S4" s="2">
         <v>0.2</v>
@@ -9059,10 +9059,10 @@
         <v>15679727</v>
       </c>
       <c r="Q5" s="1">
-        <v>67373</v>
+        <v>68554</v>
       </c>
       <c r="R5" s="1">
-        <v>2742626</v>
+        <v>2828335</v>
       </c>
       <c r="S5" s="2">
         <v>1.1</v>
@@ -9118,13 +9118,13 @@
         <v>14141465</v>
       </c>
       <c r="Q6" s="1">
-        <v>21408</v>
+        <v>23610</v>
       </c>
       <c r="R6" s="1">
-        <v>5847457</v>
+        <v>6500477</v>
       </c>
       <c r="S6" s="2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -9177,10 +9177,10 @@
         <v>12011598</v>
       </c>
       <c r="Q7" s="1">
-        <v>13679</v>
+        <v>14147</v>
       </c>
       <c r="R7" s="1">
-        <v>3446164</v>
+        <v>3552844</v>
       </c>
       <c r="S7" s="2">
         <v>1.7</v>
@@ -9236,10 +9236,10 @@
         <v>9717919</v>
       </c>
       <c r="Q8" s="1">
-        <v>42622</v>
+        <v>44641</v>
       </c>
       <c r="R8" s="1">
-        <v>2339330</v>
+        <v>2528189</v>
       </c>
       <c r="S8" s="2">
         <v>1</v>
@@ -9295,10 +9295,10 @@
         <v>9534356</v>
       </c>
       <c r="Q9" s="1">
-        <v>45592</v>
+        <v>47124</v>
       </c>
       <c r="R9" s="1">
-        <v>1760405</v>
+        <v>1829193</v>
       </c>
       <c r="S9" s="2">
         <v>1.1</v>
@@ -9354,10 +9354,10 @@
         <v>9145683</v>
       </c>
       <c r="Q10" s="1">
-        <v>64494</v>
+        <v>66050</v>
       </c>
       <c r="R10" s="1">
-        <v>1867763</v>
+        <v>2043610</v>
       </c>
       <c r="S10" s="2">
         <v>1.2</v>
@@ -9413,13 +9413,13 @@
         <v>7582485</v>
       </c>
       <c r="Q11" s="1">
-        <v>21256</v>
+        <v>22259</v>
       </c>
       <c r="R11" s="1">
-        <v>3199031</v>
+        <v>3347660</v>
       </c>
       <c r="S11" s="2">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -9472,13 +9472,13 @@
         <v>7525182</v>
       </c>
       <c r="Q12" s="1">
-        <v>39224</v>
+        <v>41334</v>
       </c>
       <c r="R12" s="1">
-        <v>3616851</v>
+        <v>3839063</v>
       </c>
       <c r="S12" s="2">
-        <v>3</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -9531,10 +9531,10 @@
         <v>7324462</v>
       </c>
       <c r="Q13" s="1">
-        <v>38832</v>
+        <v>39820</v>
       </c>
       <c r="R13" s="1">
-        <v>2748271</v>
+        <v>2851192</v>
       </c>
       <c r="S13" s="2">
         <v>1.3</v>
@@ -9590,10 +9590,10 @@
         <v>5553389</v>
       </c>
       <c r="Q14" s="1">
-        <v>33410</v>
+        <v>35058</v>
       </c>
       <c r="R14" s="1">
-        <v>1255401</v>
+        <v>1330395</v>
       </c>
       <c r="S14" s="2">
         <v>1.3</v>
@@ -9649,13 +9649,13 @@
         <v>5479176</v>
       </c>
       <c r="Q15" s="1">
-        <v>10991</v>
+        <v>11405</v>
       </c>
       <c r="R15" s="1">
-        <v>1453998</v>
+        <v>1524618</v>
       </c>
       <c r="S15" s="2">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -9708,10 +9708,10 @@
         <v>4805108</v>
       </c>
       <c r="Q16" s="1">
-        <v>6605</v>
+        <v>7315</v>
       </c>
       <c r="R16" s="1">
-        <v>802384</v>
+        <v>889693</v>
       </c>
       <c r="S16" s="2">
         <v>0.9</v>
@@ -9767,13 +9767,13 @@
         <v>4518071</v>
       </c>
       <c r="Q17" s="1">
-        <v>9527</v>
+        <v>11325</v>
       </c>
       <c r="R17" s="1">
-        <v>423606</v>
+        <v>511896</v>
       </c>
       <c r="S17" s="2">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -9826,13 +9826,13 @@
         <v>4334035</v>
       </c>
       <c r="Q18" s="1">
-        <v>6054</v>
+        <v>6425</v>
       </c>
       <c r="R18" s="1">
-        <v>920395</v>
+        <v>964848</v>
       </c>
       <c r="S18" s="2">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -9885,13 +9885,13 @@
         <v>4216981</v>
       </c>
       <c r="Q19" s="1">
-        <v>5374</v>
+        <v>5763</v>
       </c>
       <c r="R19" s="1">
-        <v>866785</v>
+        <v>926159</v>
       </c>
       <c r="S19" s="2">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -9944,13 +9944,13 @@
         <v>3849754</v>
       </c>
       <c r="Q20" s="1">
-        <v>4955</v>
+        <v>5384</v>
       </c>
       <c r="R20" s="1">
-        <v>552635</v>
+        <v>604160</v>
       </c>
       <c r="S20" s="2">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -10003,13 +10003,13 @@
         <v>3564517</v>
       </c>
       <c r="Q21" s="1">
-        <v>9202</v>
+        <v>9639</v>
       </c>
       <c r="R21" s="1">
-        <v>1361837</v>
+        <v>1440432</v>
       </c>
       <c r="S21" s="2">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -10062,10 +10062,10 @@
         <v>3485757</v>
       </c>
       <c r="Q22" s="1">
-        <v>11994</v>
+        <v>12425</v>
       </c>
       <c r="R22" s="1">
-        <v>743892</v>
+        <v>774102</v>
       </c>
       <c r="S22" s="2">
         <v>1.3</v>
@@ -10121,13 +10121,13 @@
         <v>3421998</v>
       </c>
       <c r="Q23" s="1">
-        <v>5194</v>
+        <v>6098</v>
       </c>
       <c r="R23" s="1">
-        <v>697620</v>
+        <v>768804</v>
       </c>
       <c r="S23" s="2">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -10180,13 +10180,13 @@
         <v>3403556</v>
       </c>
       <c r="Q24" s="1">
-        <v>14297</v>
+        <v>14861</v>
       </c>
       <c r="R24" s="1">
-        <v>872174</v>
+        <v>900883</v>
       </c>
       <c r="S24" s="2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -10239,13 +10239,13 @@
         <v>3153302</v>
       </c>
       <c r="Q25" s="1">
-        <v>2552</v>
+        <v>2730</v>
       </c>
       <c r="R25" s="1">
-        <v>479332</v>
+        <v>509718</v>
       </c>
       <c r="S25" s="2">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -10298,13 +10298,13 @@
         <v>2901328</v>
       </c>
       <c r="Q26" s="1">
-        <v>10910</v>
+        <v>11285</v>
       </c>
       <c r="R26" s="1">
-        <v>985591</v>
+        <v>1029298</v>
       </c>
       <c r="S26" s="2">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="27" spans="1:19">
@@ -10357,13 +10357,13 @@
         <v>2127393</v>
       </c>
       <c r="Q27" s="1">
-        <v>5439</v>
+        <v>5943</v>
       </c>
       <c r="R27" s="1">
-        <v>408169</v>
+        <v>459278</v>
       </c>
       <c r="S27" s="2">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="28" spans="1:19">
@@ -10416,13 +10416,13 @@
         <v>2051386</v>
       </c>
       <c r="Q28" s="1">
-        <v>5479</v>
+        <v>5862</v>
       </c>
       <c r="R28" s="1">
-        <v>581868</v>
+        <v>633268</v>
       </c>
       <c r="S28" s="2">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="29" spans="1:19">
@@ -10475,10 +10475,10 @@
         <v>1996475</v>
       </c>
       <c r="Q29" s="1">
-        <v>3311</v>
+        <v>3224</v>
       </c>
       <c r="R29" s="1">
-        <v>536163</v>
+        <v>537945</v>
       </c>
       <c r="S29" s="2">
         <v>1.6</v>
@@ -10534,13 +10534,13 @@
         <v>1992220</v>
       </c>
       <c r="Q30" s="1">
-        <v>3699</v>
+        <v>4013</v>
       </c>
       <c r="R30" s="1">
-        <v>601826</v>
+        <v>637402</v>
       </c>
       <c r="S30" s="2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="31" spans="1:19">
@@ -10593,13 +10593,13 @@
         <v>1952923</v>
       </c>
       <c r="Q31" s="1">
-        <v>1607</v>
+        <v>2225</v>
       </c>
       <c r="R31" s="1">
-        <v>185280</v>
+        <v>252307</v>
       </c>
       <c r="S31" s="2">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="32" spans="1:19">
@@ -10652,13 +10652,13 @@
         <v>1830717</v>
       </c>
       <c r="Q32" s="1">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="R32" s="1">
-        <v>34284</v>
+        <v>38277</v>
       </c>
       <c r="S32" s="2">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="33" spans="1:19">
@@ -10711,13 +10711,13 @@
         <v>1729934</v>
       </c>
       <c r="Q33" s="1">
-        <v>4880</v>
+        <v>4959</v>
       </c>
       <c r="R33" s="1">
-        <v>956119</v>
+        <v>985941</v>
       </c>
       <c r="S33" s="2">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="34" spans="1:19">
@@ -10770,10 +10770,10 @@
         <v>1719805</v>
       </c>
       <c r="Q34" s="1">
-        <v>10208</v>
+        <v>10934</v>
       </c>
       <c r="R34" s="1">
-        <v>283499</v>
+        <v>323928</v>
       </c>
       <c r="S34" s="2">
         <v>0.8</v>
@@ -10829,13 +10829,13 @@
         <v>1717791</v>
       </c>
       <c r="Q35" s="1">
-        <v>6740</v>
+        <v>8101</v>
       </c>
       <c r="R35" s="1">
-        <v>175784</v>
+        <v>205375</v>
       </c>
       <c r="S35" s="2">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="36" spans="1:19">
@@ -10888,13 +10888,13 @@
         <v>1710906</v>
       </c>
       <c r="Q36" s="1">
-        <v>4336</v>
+        <v>4463</v>
       </c>
       <c r="R36" s="1">
-        <v>419804</v>
+        <v>432534</v>
       </c>
       <c r="S36" s="2">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="37" spans="1:19">
@@ -10947,13 +10947,13 @@
         <v>1633719</v>
       </c>
       <c r="Q37" s="1">
-        <v>6928</v>
+        <v>7279</v>
       </c>
       <c r="R37" s="1">
-        <v>318090</v>
+        <v>332080</v>
       </c>
       <c r="S37" s="2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="38" spans="1:19">
@@ -11006,10 +11006,10 @@
         <v>1613859</v>
       </c>
       <c r="Q38" s="1">
-        <v>6000</v>
+        <v>6022</v>
       </c>
       <c r="R38" s="1">
-        <v>743384</v>
+        <v>746454</v>
       </c>
       <c r="S38" s="2">
         <v>2.4</v>
@@ -11065,13 +11065,13 @@
         <v>1548859</v>
       </c>
       <c r="Q39" s="1">
-        <v>1438</v>
+        <v>1620</v>
       </c>
       <c r="R39" s="1">
-        <v>374317</v>
+        <v>424966</v>
       </c>
       <c r="S39" s="2">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="40" spans="1:19">
@@ -11124,13 +11124,13 @@
         <v>1541969</v>
       </c>
       <c r="Q40" s="1">
-        <v>928</v>
+        <v>1373</v>
       </c>
       <c r="R40" s="1">
-        <v>105418</v>
+        <v>156825</v>
       </c>
       <c r="S40" s="2">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="41" spans="1:19">
@@ -11183,13 +11183,13 @@
         <v>1536754</v>
       </c>
       <c r="Q41" s="1">
-        <v>1395</v>
+        <v>1647</v>
       </c>
       <c r="R41" s="1">
-        <v>411284</v>
+        <v>491474</v>
       </c>
       <c r="S41" s="2">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="42" spans="1:19">
@@ -11242,13 +11242,13 @@
         <v>1502872</v>
       </c>
       <c r="Q42" s="1">
-        <v>1084</v>
+        <v>1217</v>
       </c>
       <c r="R42" s="1">
-        <v>209801</v>
+        <v>246815</v>
       </c>
       <c r="S42" s="2">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="43" spans="1:19">
@@ -11301,10 +11301,10 @@
         <v>1414849</v>
       </c>
       <c r="Q43" s="1">
-        <v>9391</v>
+        <v>9920</v>
       </c>
       <c r="R43" s="1">
-        <v>275777</v>
+        <v>309308</v>
       </c>
       <c r="S43" s="2">
         <v>0.8</v>
@@ -11360,13 +11360,13 @@
         <v>1365547</v>
       </c>
       <c r="Q44" s="1">
-        <v>2932</v>
+        <v>3112</v>
       </c>
       <c r="R44" s="1">
-        <v>658564</v>
+        <v>706473</v>
       </c>
       <c r="S44" s="2">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="45" spans="1:19">
@@ -11419,10 +11419,10 @@
         <v>1258947</v>
       </c>
       <c r="Q45" s="1">
-        <v>11860</v>
+        <v>12000</v>
       </c>
       <c r="R45" s="1">
-        <v>368280</v>
+        <v>374813</v>
       </c>
       <c r="S45" s="2">
         <v>1.6</v>
@@ -11478,13 +11478,13 @@
         <v>1222686</v>
       </c>
       <c r="Q46" s="1">
-        <v>4836</v>
+        <v>5134</v>
       </c>
       <c r="R46" s="1">
-        <v>211227</v>
+        <v>224587</v>
       </c>
       <c r="S46" s="2">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="47" spans="1:19">
@@ -11537,13 +11537,13 @@
         <v>1200781</v>
       </c>
       <c r="Q47" s="1">
-        <v>9660</v>
+        <v>11440</v>
       </c>
       <c r="R47" s="1">
-        <v>323964</v>
+        <v>366010</v>
       </c>
       <c r="S47" s="2">
-        <v>1.7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:19">
@@ -11596,10 +11596,10 @@
         <v>1168782</v>
       </c>
       <c r="Q48" s="1">
-        <v>4165</v>
+        <v>4195</v>
       </c>
       <c r="R48" s="1">
-        <v>425752</v>
+        <v>429023</v>
       </c>
       <c r="S48" s="2">
         <v>2</v>
@@ -11714,10 +11714,10 @@
         <v>1053912</v>
       </c>
       <c r="Q50" s="1">
-        <v>2537</v>
+        <v>2556</v>
       </c>
       <c r="R50" s="1">
-        <v>296371</v>
+        <v>297945</v>
       </c>
       <c r="S50" s="2">
         <v>1.4</v>
@@ -11773,13 +11773,13 @@
         <v>962277</v>
       </c>
       <c r="Q51" s="1">
-        <v>6065</v>
+        <v>6250</v>
       </c>
       <c r="R51" s="1">
-        <v>687010</v>
+        <v>719335</v>
       </c>
       <c r="S51" s="2">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="52" spans="1:19">
@@ -11832,13 +11832,13 @@
         <v>938957</v>
       </c>
       <c r="Q52" s="1">
-        <v>1761</v>
+        <v>2116</v>
       </c>
       <c r="R52" s="1">
-        <v>75983</v>
+        <v>102159</v>
       </c>
       <c r="S52" s="2">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="53" spans="1:19">
@@ -11891,10 +11891,10 @@
         <v>917414</v>
       </c>
       <c r="Q53" s="1">
-        <v>1221</v>
+        <v>1237</v>
       </c>
       <c r="R53" s="1">
-        <v>180051</v>
+        <v>182947</v>
       </c>
       <c r="S53" s="2">
         <v>1.1</v>
@@ -11950,13 +11950,13 @@
         <v>869605</v>
       </c>
       <c r="Q54" s="1">
-        <v>1050</v>
+        <v>1201</v>
       </c>
       <c r="R54" s="1">
-        <v>314412</v>
+        <v>364427</v>
       </c>
       <c r="S54" s="2">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:19">
@@ -12009,13 +12009,13 @@
         <v>865930</v>
       </c>
       <c r="Q55" s="1">
-        <v>1500</v>
+        <v>1542</v>
       </c>
       <c r="R55" s="1">
-        <v>318152</v>
+        <v>332104</v>
       </c>
       <c r="S55" s="2">
-        <v>1.9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:19">
@@ -12068,10 +12068,10 @@
         <v>795798</v>
       </c>
       <c r="Q56" s="1">
-        <v>889</v>
+        <v>880</v>
       </c>
       <c r="R56" s="1">
-        <v>300454</v>
+        <v>302103</v>
       </c>
       <c r="S56" s="2">
         <v>1.6</v>
@@ -12127,13 +12127,13 @@
         <v>771123</v>
       </c>
       <c r="Q57" s="1">
-        <v>1082</v>
+        <v>1128</v>
       </c>
       <c r="R57" s="1">
-        <v>424549</v>
+        <v>444020</v>
       </c>
       <c r="S57" s="2">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="58" spans="1:19">
@@ -12186,10 +12186,10 @@
         <v>770501</v>
       </c>
       <c r="Q58" s="1">
-        <v>2568</v>
+        <v>2623</v>
       </c>
       <c r="R58" s="1">
-        <v>221379</v>
+        <v>225934</v>
       </c>
       <c r="S58" s="2">
         <v>1.5</v>
@@ -12245,10 +12245,10 @@
         <v>725876</v>
       </c>
       <c r="Q59" s="1">
-        <v>9399</v>
+        <v>9538</v>
       </c>
       <c r="R59" s="1">
-        <v>499040</v>
+        <v>505640</v>
       </c>
       <c r="S59" s="2">
         <v>4.2</v>
@@ -12304,13 +12304,13 @@
         <v>705719</v>
       </c>
       <c r="Q60" s="1">
-        <v>4839</v>
+        <v>5139</v>
       </c>
       <c r="R60" s="1">
-        <v>342558</v>
+        <v>365301</v>
       </c>
       <c r="S60" s="2">
-        <v>2.8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61" spans="1:19">
@@ -12363,10 +12363,10 @@
         <v>698835</v>
       </c>
       <c r="Q61" s="1">
-        <v>1881</v>
+        <v>1902</v>
       </c>
       <c r="R61" s="1">
-        <v>150430</v>
+        <v>151898</v>
       </c>
       <c r="S61" s="2">
         <v>1.3</v>
@@ -12422,13 +12422,13 @@
         <v>587724</v>
       </c>
       <c r="Q62" s="1">
-        <v>2863</v>
+        <v>4372</v>
       </c>
       <c r="R62" s="1">
-        <v>81353</v>
+        <v>114338</v>
       </c>
       <c r="S62" s="2">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="63" spans="1:19">
@@ -12540,10 +12540,10 @@
         <v>576776</v>
       </c>
       <c r="Q64" s="1">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="R64" s="1">
-        <v>104280</v>
+        <v>105850</v>
       </c>
       <c r="S64" s="2">
         <v>1.2</v>
@@ -12599,13 +12599,13 @@
         <v>569994</v>
       </c>
       <c r="Q65" s="1">
-        <v>1126</v>
+        <v>1187</v>
       </c>
       <c r="R65" s="1">
-        <v>279014</v>
+        <v>284460</v>
       </c>
       <c r="S65" s="2">
-        <v>2.4</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="66" spans="1:19">
@@ -12658,13 +12658,13 @@
         <v>543885</v>
       </c>
       <c r="Q66" s="1">
-        <v>574</v>
+        <v>606</v>
       </c>
       <c r="R66" s="1">
-        <v>93006</v>
+        <v>100035</v>
       </c>
       <c r="S66" s="2">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:19">
@@ -12717,13 +12717,13 @@
         <v>525089</v>
       </c>
       <c r="Q67" s="1">
-        <v>807</v>
+        <v>823</v>
       </c>
       <c r="R67" s="1">
-        <v>160586</v>
+        <v>170585</v>
       </c>
       <c r="S67" s="2">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="68" spans="1:19">
@@ -12776,13 +12776,13 @@
         <v>507215</v>
       </c>
       <c r="Q68" s="1">
-        <v>999</v>
+        <v>1084</v>
       </c>
       <c r="R68" s="1">
-        <v>78063</v>
+        <v>87308</v>
       </c>
       <c r="S68" s="2">
-        <v>0.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:19">
@@ -12835,13 +12835,13 @@
         <v>506044</v>
       </c>
       <c r="Q69" s="1">
-        <v>17344</v>
+        <v>17552</v>
       </c>
       <c r="R69" s="1">
-        <v>845962</v>
+        <v>847060</v>
       </c>
       <c r="S69" s="2">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="70" spans="1:19">
@@ -12894,13 +12894,13 @@
         <v>503475</v>
       </c>
       <c r="Q70" s="1">
-        <v>3691</v>
+        <v>4729</v>
       </c>
       <c r="R70" s="1">
-        <v>424583</v>
+        <v>590344</v>
       </c>
       <c r="S70" s="2">
-        <v>4</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="71" spans="1:19">
@@ -12953,10 +12953,10 @@
         <v>494215</v>
       </c>
       <c r="Q71" s="1">
-        <v>2182</v>
+        <v>2169</v>
       </c>
       <c r="R71" s="1">
-        <v>60487</v>
+        <v>82913</v>
       </c>
       <c r="S71" s="2">
         <v>0.7</v>
@@ -13012,13 +13012,13 @@
         <v>481799</v>
       </c>
       <c r="Q72" s="1">
-        <v>1927</v>
+        <v>2087</v>
       </c>
       <c r="R72" s="1">
-        <v>126025</v>
+        <v>135680</v>
       </c>
       <c r="S72" s="2">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="73" spans="1:19">
@@ -13071,13 +13071,13 @@
         <v>446545</v>
       </c>
       <c r="Q73" s="1">
-        <v>2379</v>
+        <v>2700</v>
       </c>
       <c r="R73" s="1">
-        <v>204901</v>
+        <v>228614</v>
       </c>
       <c r="S73" s="2">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="74" spans="1:19">
@@ -13130,13 +13130,13 @@
         <v>443725</v>
       </c>
       <c r="Q74" s="1">
-        <v>866</v>
+        <v>926</v>
       </c>
       <c r="R74" s="1">
-        <v>80986</v>
+        <v>84293</v>
       </c>
       <c r="S74" s="2">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="75" spans="1:19">
@@ -13189,10 +13189,10 @@
         <v>419678</v>
       </c>
       <c r="Q75" s="1">
-        <v>3280</v>
+        <v>3336</v>
       </c>
       <c r="R75" s="1">
-        <v>315608</v>
+        <v>328466</v>
       </c>
       <c r="S75" s="2">
         <v>2.2</v>
@@ -13248,13 +13248,13 @@
         <v>416146</v>
       </c>
       <c r="Q76" s="1">
-        <v>526</v>
+        <v>552</v>
       </c>
       <c r="R76" s="1">
-        <v>321039</v>
+        <v>325689</v>
       </c>
       <c r="S76" s="2">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="77" spans="1:19">
@@ -13307,13 +13307,13 @@
         <v>399232</v>
       </c>
       <c r="Q77" s="1">
-        <v>3386</v>
+        <v>3056</v>
       </c>
       <c r="R77" s="1">
-        <v>145090</v>
+        <v>145900</v>
       </c>
       <c r="S77" s="2">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="78" spans="1:19">
@@ -13366,13 +13366,13 @@
         <v>371222</v>
       </c>
       <c r="Q78" s="1">
-        <v>3480</v>
+        <v>3560</v>
       </c>
       <c r="R78" s="1">
-        <v>533698</v>
+        <v>542018</v>
       </c>
       <c r="S78" s="2">
-        <v>6.1</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="79" spans="1:19">
@@ -13425,13 +13425,13 @@
         <v>367850</v>
       </c>
       <c r="Q79" s="1">
-        <v>1591</v>
+        <v>1618</v>
       </c>
       <c r="R79" s="1">
-        <v>142194</v>
+        <v>147283</v>
       </c>
       <c r="S79" s="2">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="80" spans="1:19">
@@ -13484,13 +13484,13 @@
         <v>363780</v>
       </c>
       <c r="Q80" s="1">
-        <v>3243</v>
+        <v>3293</v>
       </c>
       <c r="R80" s="1">
-        <v>360614</v>
+        <v>365008</v>
       </c>
       <c r="S80" s="2">
-        <v>6</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="81" spans="1:19">
@@ -13543,10 +13543,10 @@
         <v>356405</v>
       </c>
       <c r="Q81" s="1">
-        <v>980</v>
+        <v>975</v>
       </c>
       <c r="R81" s="1">
-        <v>85098</v>
+        <v>85170</v>
       </c>
       <c r="S81" s="2">
         <v>1.5</v>
@@ -13602,10 +13602,10 @@
         <v>353335</v>
       </c>
       <c r="Q82" s="1">
-        <v>1586</v>
+        <v>1598</v>
       </c>
       <c r="R82" s="1">
-        <v>164614</v>
+        <v>165988</v>
       </c>
       <c r="S82" s="2">
         <v>2.7</v>
@@ -13661,13 +13661,13 @@
         <v>335048</v>
       </c>
       <c r="Q83" s="1">
-        <v>1589</v>
+        <v>1717</v>
       </c>
       <c r="R83" s="1">
-        <v>143454</v>
+        <v>155882</v>
       </c>
       <c r="S83" s="2">
-        <v>3</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="84" spans="1:19">
@@ -13720,10 +13720,10 @@
         <v>324792</v>
       </c>
       <c r="Q84" s="1">
-        <v>3534</v>
+        <v>3552</v>
       </c>
       <c r="R84" s="1">
-        <v>249542</v>
+        <v>251520</v>
       </c>
       <c r="S84" s="2">
         <v>4.4</v>
@@ -13779,10 +13779,10 @@
         <v>312069</v>
       </c>
       <c r="Q85" s="1">
-        <v>1805</v>
+        <v>1887</v>
       </c>
       <c r="R85" s="1">
-        <v>112586</v>
+        <v>115063</v>
       </c>
       <c r="S85" s="2">
         <v>1</v>
@@ -13838,10 +13838,10 @@
         <v>306511</v>
       </c>
       <c r="Q86" s="1">
-        <v>852</v>
+        <v>887</v>
       </c>
       <c r="R86" s="1">
-        <v>77956</v>
+        <v>82365</v>
       </c>
       <c r="S86" s="2">
         <v>1.2</v>
@@ -13897,13 +13897,13 @@
         <v>306374</v>
       </c>
       <c r="Q87" s="1">
-        <v>927</v>
+        <v>956</v>
       </c>
       <c r="R87" s="1">
-        <v>92476</v>
+        <v>95158</v>
       </c>
       <c r="S87" s="2">
-        <v>1.9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:19">
@@ -13956,10 +13956,10 @@
         <v>303328</v>
       </c>
       <c r="Q88" s="1">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="R88" s="1">
-        <v>6000</v>
+        <v>6152</v>
       </c>
       <c r="S88" s="2">
         <v>0.1</v>
@@ -14015,7 +14015,7 @@
         <v>287372</v>
       </c>
       <c r="Q89" s="1">
-        <v>1324</v>
+        <v>1314</v>
       </c>
       <c r="R89" s="1">
         <v>182207</v>
@@ -14074,10 +14074,10 @@
         <v>279120</v>
       </c>
       <c r="Q90" s="1">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="R90" s="1">
-        <v>7126</v>
+        <v>7441</v>
       </c>
       <c r="S90" s="2">
         <v>0.2</v>
@@ -14133,13 +14133,13 @@
         <v>258797</v>
       </c>
       <c r="Q91" s="1">
-        <v>751</v>
+        <v>871</v>
       </c>
       <c r="R91" s="1">
-        <v>53938</v>
+        <v>62770</v>
       </c>
       <c r="S91" s="2">
-        <v>1.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="92" spans="1:19">
@@ -14192,13 +14192,13 @@
         <v>257112</v>
       </c>
       <c r="Q92" s="1">
-        <v>374</v>
+        <v>623</v>
       </c>
       <c r="R92" s="1">
-        <v>69212</v>
+        <v>98854</v>
       </c>
       <c r="S92" s="2">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="93" spans="1:19">
@@ -14251,10 +14251,10 @@
         <v>247853</v>
       </c>
       <c r="Q93" s="1">
-        <v>5678</v>
+        <v>5680</v>
       </c>
       <c r="R93" s="1">
-        <v>824852</v>
+        <v>824972</v>
       </c>
       <c r="S93" s="2">
         <v>11.4</v>
@@ -14310,13 +14310,13 @@
         <v>247507</v>
       </c>
       <c r="Q94" s="1">
-        <v>610</v>
+        <v>603</v>
       </c>
       <c r="R94" s="1">
-        <v>101210</v>
+        <v>102296</v>
       </c>
       <c r="S94" s="2">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="95" spans="1:19">
@@ -14369,13 +14369,13 @@
         <v>232232</v>
       </c>
       <c r="Q95" s="1">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="R95" s="1">
-        <v>9155</v>
+        <v>18737</v>
       </c>
       <c r="S95" s="2">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="96" spans="1:19">
@@ -14428,13 +14428,13 @@
         <v>228869</v>
       </c>
       <c r="Q96" s="1">
-        <v>834</v>
+        <v>959</v>
       </c>
       <c r="R96" s="1">
-        <v>53338</v>
+        <v>61533</v>
       </c>
       <c r="S96" s="2">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="97" spans="1:19">
@@ -14487,13 +14487,13 @@
         <v>222516</v>
       </c>
       <c r="Q97" s="1">
-        <v>4748</v>
+        <v>4873</v>
       </c>
       <c r="R97" s="1">
-        <v>565737</v>
+        <v>582922</v>
       </c>
       <c r="S97" s="2">
-        <v>11.7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="98" spans="1:19">
@@ -14546,10 +14546,10 @@
         <v>209820</v>
       </c>
       <c r="Q98" s="1">
-        <v>3478</v>
+        <v>3500</v>
       </c>
       <c r="R98" s="1">
-        <v>188378</v>
+        <v>189934</v>
       </c>
       <c r="S98" s="2">
         <v>5.7</v>
@@ -14605,10 +14605,10 @@
         <v>205272</v>
       </c>
       <c r="Q99" s="1">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="R99" s="1">
-        <v>122694</v>
+        <v>123683</v>
       </c>
       <c r="S99" s="2">
         <v>2.7</v>
@@ -14664,13 +14664,13 @@
         <v>192351</v>
       </c>
       <c r="Q100" s="1">
-        <v>1439</v>
+        <v>1500</v>
       </c>
       <c r="R100" s="1">
-        <v>320059</v>
+        <v>339352</v>
       </c>
       <c r="S100" s="2">
-        <v>10.9</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="101" spans="1:19">
@@ -14723,10 +14723,10 @@
         <v>188616</v>
       </c>
       <c r="Q101" s="1">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="R101" s="1">
-        <v>58343</v>
+        <v>58593</v>
       </c>
       <c r="S101" s="2">
         <v>1.8</v>
@@ -14782,13 +14782,13 @@
         <v>181446</v>
       </c>
       <c r="Q102" s="1">
-        <v>1773</v>
+        <v>1816</v>
       </c>
       <c r="R102" s="1">
-        <v>112606</v>
+        <v>117499</v>
       </c>
       <c r="S102" s="2">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="103" spans="1:19">
@@ -14900,13 +14900,13 @@
         <v>166081</v>
       </c>
       <c r="Q104" s="1">
-        <v>1273</v>
+        <v>1301</v>
       </c>
       <c r="R104" s="1">
-        <v>111075</v>
+        <v>115680</v>
       </c>
       <c r="S104" s="2">
-        <v>2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="105" spans="1:19">
@@ -14959,10 +14959,10 @@
         <v>165708</v>
       </c>
       <c r="Q105" s="1">
-        <v>505</v>
+        <v>526</v>
       </c>
       <c r="R105" s="1">
-        <v>25766</v>
+        <v>26563</v>
       </c>
       <c r="S105" s="2">
         <v>0.9</v>
@@ -15018,13 +15018,13 @@
         <v>162658</v>
       </c>
       <c r="Q106" s="1">
-        <v>2464</v>
+        <v>2785</v>
       </c>
       <c r="R106" s="1">
-        <v>78163</v>
+        <v>84261</v>
       </c>
       <c r="S106" s="2">
-        <v>2.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="107" spans="1:19">
@@ -15077,10 +15077,10 @@
         <v>160758</v>
       </c>
       <c r="Q107" s="1">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="R107" s="1">
-        <v>119198</v>
+        <v>119460</v>
       </c>
       <c r="S107" s="2">
         <v>4.4</v>
@@ -15136,13 +15136,13 @@
         <v>155919</v>
       </c>
       <c r="Q108" s="1">
-        <v>1234</v>
+        <v>1332</v>
       </c>
       <c r="R108" s="1">
-        <v>52432</v>
+        <v>56555</v>
       </c>
       <c r="S108" s="2">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="109" spans="1:19">
@@ -15195,10 +15195,10 @@
         <v>145054</v>
       </c>
       <c r="Q109" s="1">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="R109" s="1">
-        <v>118606</v>
+        <v>120437</v>
       </c>
       <c r="S109" s="2">
         <v>3.3</v>
@@ -15254,10 +15254,10 @@
         <v>125380</v>
       </c>
       <c r="Q110" s="1">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="R110" s="1">
-        <v>36241</v>
+        <v>37981</v>
       </c>
       <c r="S110" s="2">
         <v>1.7</v>
@@ -15313,10 +15313,10 @@
         <v>119439</v>
       </c>
       <c r="Q111" s="1">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="R111" s="1">
-        <v>36775</v>
+        <v>36824</v>
       </c>
       <c r="S111" s="2">
         <v>1.8</v>
@@ -15431,13 +15431,13 @@
         <v>108899</v>
       </c>
       <c r="Q113" s="1">
-        <v>416</v>
+        <v>462</v>
       </c>
       <c r="R113" s="1">
-        <v>21236</v>
+        <v>23593</v>
       </c>
       <c r="S113" s="2">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="114" spans="1:19">
@@ -15490,13 +15490,13 @@
         <v>85756</v>
       </c>
       <c r="Q114" s="1">
-        <v>79</v>
+        <v>192</v>
       </c>
       <c r="R114" s="1">
-        <v>5286</v>
+        <v>17455</v>
       </c>
       <c r="S114" s="2">
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:19">
@@ -15549,10 +15549,10 @@
         <v>77595</v>
       </c>
       <c r="Q115" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R115" s="1">
-        <v>258</v>
+        <v>295</v>
       </c>
       <c r="S115" s="2">
         <v>0</v>
@@ -15667,10 +15667,10 @@
         <v>70476</v>
       </c>
       <c r="Q117" s="1">
-        <v>422</v>
+        <v>442</v>
       </c>
       <c r="R117" s="1">
-        <v>13014</v>
+        <v>13614</v>
       </c>
       <c r="S117" s="2">
         <v>1.1</v>
@@ -15726,13 +15726,13 @@
         <v>65173</v>
       </c>
       <c r="Q118" s="1">
-        <v>261</v>
+        <v>387</v>
       </c>
       <c r="R118" s="1">
-        <v>19109</v>
+        <v>26053</v>
       </c>
       <c r="S118" s="2">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="119" spans="1:19">
@@ -15785,13 +15785,13 @@
         <v>61440</v>
       </c>
       <c r="Q119" s="1">
-        <v>166</v>
+        <v>258</v>
       </c>
       <c r="R119" s="1">
-        <v>7950</v>
+        <v>10610</v>
       </c>
       <c r="S119" s="2">
-        <v>0.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120" spans="1:19">
@@ -15962,13 +15962,13 @@
         <v>36954</v>
       </c>
       <c r="Q122" s="1">
-        <v>2186</v>
+        <v>2263</v>
       </c>
       <c r="R122" s="1">
-        <v>64866</v>
+        <v>67176</v>
       </c>
       <c r="S122" s="2">
-        <v>10.6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="123" spans="1:19">
@@ -16021,13 +16021,13 @@
         <v>34286</v>
       </c>
       <c r="Q123" s="1">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="R123" s="1">
-        <v>33271</v>
+        <v>33886</v>
       </c>
       <c r="S123" s="2">
-        <v>5.8</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="124" spans="1:19">
@@ -16080,10 +16080,10 @@
         <v>30897</v>
       </c>
       <c r="Q124" s="1">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="R124" s="1">
-        <v>10353</v>
+        <v>10473</v>
       </c>
       <c r="S124" s="2">
         <v>0</v>
@@ -16139,10 +16139,10 @@
         <v>25268</v>
       </c>
       <c r="Q125" s="1">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="R125" s="1">
-        <v>9791</v>
+        <v>9855</v>
       </c>
       <c r="S125" s="2">
         <v>2.5</v>
@@ -16257,13 +16257,13 @@
         <v>2439</v>
       </c>
       <c r="Q127" s="1">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="R127" s="1">
-        <v>1347</v>
+        <v>2089</v>
       </c>
       <c r="S127" s="2">
-        <v>3.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="128" spans="1:19">
@@ -16375,13 +16375,13 @@
         <v>94</v>
       </c>
       <c r="Q129" s="1">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="R129" s="1">
-        <v>1030</v>
+        <v>1201</v>
       </c>
       <c r="S129" s="2">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="130" spans="1:19">
@@ -16434,10 +16434,10 @@
         <v>0</v>
       </c>
       <c r="Q130" s="1">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="R130" s="1">
-        <v>1102</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="131" spans="1:19">
@@ -16546,10 +16546,10 @@
         <v>0</v>
       </c>
       <c r="Q132" s="1">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R132" s="1">
-        <v>40</v>
+        <v>556</v>
       </c>
     </row>
     <row r="133" spans="1:19">

</xml_diff>

<commit_message>
Use All Items sheet for stock values in full Gujarat supplier-wise report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016DwJnqVusC3tRSWnF3Qvwz
</commit_message>
<xml_diff>
--- a/docs/Supplier_wise_Full_GJ.xlsx
+++ b/docs/Supplier_wise_Full_GJ.xlsx
@@ -1370,13 +1370,13 @@
         <v>54255889</v>
       </c>
       <c r="P2" s="1">
-        <v>303751</v>
+        <v>282991</v>
       </c>
       <c r="Q2" s="1">
-        <v>25252505</v>
+        <v>23708597</v>
       </c>
       <c r="R2" s="2">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="S2" s="1" t="s">
         <v>145</v>
@@ -1429,13 +1429,13 @@
         <v>45524507</v>
       </c>
       <c r="P3" s="1">
-        <v>136428</v>
+        <v>129700</v>
       </c>
       <c r="Q3" s="1">
-        <v>24486238</v>
+        <v>23338272</v>
       </c>
       <c r="R3" s="2">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="S3" s="1" t="s">
         <v>146</v>
@@ -1488,10 +1488,10 @@
         <v>20240180</v>
       </c>
       <c r="P4" s="1">
-        <v>12837</v>
+        <v>12140</v>
       </c>
       <c r="Q4" s="1">
-        <v>1223754</v>
+        <v>1137858</v>
       </c>
       <c r="R4" s="2">
         <v>0.2</v>
@@ -1547,10 +1547,10 @@
         <v>15679727</v>
       </c>
       <c r="P5" s="1">
-        <v>68554</v>
+        <v>67373</v>
       </c>
       <c r="Q5" s="1">
-        <v>2828335</v>
+        <v>2742626</v>
       </c>
       <c r="R5" s="2">
         <v>1.1</v>
@@ -1606,13 +1606,13 @@
         <v>14141465</v>
       </c>
       <c r="P6" s="1">
-        <v>23610</v>
+        <v>21408</v>
       </c>
       <c r="Q6" s="1">
-        <v>6500477</v>
+        <v>5847457</v>
       </c>
       <c r="R6" s="2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="S6" s="1" t="s">
         <v>149</v>
@@ -1665,10 +1665,10 @@
         <v>12011598</v>
       </c>
       <c r="P7" s="1">
-        <v>14147</v>
+        <v>13679</v>
       </c>
       <c r="Q7" s="1">
-        <v>3552844</v>
+        <v>3446164</v>
       </c>
       <c r="R7" s="2">
         <v>1.7</v>
@@ -1724,10 +1724,10 @@
         <v>9717919</v>
       </c>
       <c r="P8" s="1">
-        <v>44641</v>
+        <v>42622</v>
       </c>
       <c r="Q8" s="1">
-        <v>2528189</v>
+        <v>2339330</v>
       </c>
       <c r="R8" s="2">
         <v>1</v>
@@ -1783,10 +1783,10 @@
         <v>9534356</v>
       </c>
       <c r="P9" s="1">
-        <v>47124</v>
+        <v>45592</v>
       </c>
       <c r="Q9" s="1">
-        <v>1829193</v>
+        <v>1760405</v>
       </c>
       <c r="R9" s="2">
         <v>1.1</v>
@@ -1842,10 +1842,10 @@
         <v>9145683</v>
       </c>
       <c r="P10" s="1">
-        <v>66050</v>
+        <v>64494</v>
       </c>
       <c r="Q10" s="1">
-        <v>2043610</v>
+        <v>1867763</v>
       </c>
       <c r="R10" s="2">
         <v>1.2</v>
@@ -1901,13 +1901,13 @@
         <v>7717533</v>
       </c>
       <c r="P11" s="1">
-        <v>42834</v>
+        <v>40663</v>
       </c>
       <c r="Q11" s="1">
-        <v>4178415</v>
+        <v>3936910</v>
       </c>
       <c r="R11" s="2">
-        <v>3.2</v>
+        <v>3.1</v>
       </c>
       <c r="S11" s="1" t="s">
         <v>154</v>
@@ -1960,13 +1960,13 @@
         <v>7582485</v>
       </c>
       <c r="P12" s="1">
-        <v>22259</v>
+        <v>21256</v>
       </c>
       <c r="Q12" s="1">
-        <v>3347660</v>
+        <v>3199031</v>
       </c>
       <c r="R12" s="2">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="S12" s="1" t="s">
         <v>155</v>
@@ -2019,10 +2019,10 @@
         <v>7324462</v>
       </c>
       <c r="P13" s="1">
-        <v>39820</v>
+        <v>38832</v>
       </c>
       <c r="Q13" s="1">
-        <v>2851192</v>
+        <v>2748271</v>
       </c>
       <c r="R13" s="2">
         <v>1.3</v>
@@ -2078,10 +2078,10 @@
         <v>5553389</v>
       </c>
       <c r="P14" s="1">
-        <v>35058</v>
+        <v>33410</v>
       </c>
       <c r="Q14" s="1">
-        <v>1330395</v>
+        <v>1255401</v>
       </c>
       <c r="R14" s="2">
         <v>1.3</v>
@@ -2137,13 +2137,13 @@
         <v>5479176</v>
       </c>
       <c r="P15" s="1">
-        <v>11405</v>
+        <v>10991</v>
       </c>
       <c r="Q15" s="1">
-        <v>1524618</v>
+        <v>1453998</v>
       </c>
       <c r="R15" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="S15" s="1" t="s">
         <v>158</v>
@@ -2196,10 +2196,10 @@
         <v>4805108</v>
       </c>
       <c r="P16" s="1">
-        <v>7315</v>
+        <v>6605</v>
       </c>
       <c r="Q16" s="1">
-        <v>889693</v>
+        <v>802384</v>
       </c>
       <c r="R16" s="2">
         <v>0.9</v>
@@ -2255,13 +2255,13 @@
         <v>4518071</v>
       </c>
       <c r="P17" s="1">
-        <v>11325</v>
+        <v>9527</v>
       </c>
       <c r="Q17" s="1">
-        <v>511896</v>
+        <v>423606</v>
       </c>
       <c r="R17" s="2">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="S17" s="1" t="s">
         <v>160</v>
@@ -2314,13 +2314,13 @@
         <v>4334035</v>
       </c>
       <c r="P18" s="1">
-        <v>6425</v>
+        <v>6054</v>
       </c>
       <c r="Q18" s="1">
-        <v>964848</v>
+        <v>920395</v>
       </c>
       <c r="R18" s="2">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="S18" s="1" t="s">
         <v>161</v>
@@ -2373,13 +2373,13 @@
         <v>4216981</v>
       </c>
       <c r="P19" s="1">
-        <v>5763</v>
+        <v>5374</v>
       </c>
       <c r="Q19" s="1">
-        <v>926159</v>
+        <v>866785</v>
       </c>
       <c r="R19" s="2">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="S19" s="1" t="s">
         <v>162</v>
@@ -2432,13 +2432,13 @@
         <v>3849754</v>
       </c>
       <c r="P20" s="1">
-        <v>5384</v>
+        <v>4955</v>
       </c>
       <c r="Q20" s="1">
-        <v>604160</v>
+        <v>552635</v>
       </c>
       <c r="R20" s="2">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="S20" s="1" t="s">
         <v>163</v>
@@ -2491,13 +2491,13 @@
         <v>3564517</v>
       </c>
       <c r="P21" s="1">
-        <v>9639</v>
+        <v>9202</v>
       </c>
       <c r="Q21" s="1">
-        <v>1440432</v>
+        <v>1361837</v>
       </c>
       <c r="R21" s="2">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="S21" s="1" t="s">
         <v>164</v>
@@ -2550,10 +2550,10 @@
         <v>3485757</v>
       </c>
       <c r="P22" s="1">
-        <v>12425</v>
+        <v>11994</v>
       </c>
       <c r="Q22" s="1">
-        <v>774102</v>
+        <v>743892</v>
       </c>
       <c r="R22" s="2">
         <v>1.3</v>
@@ -2609,13 +2609,13 @@
         <v>3421998</v>
       </c>
       <c r="P23" s="1">
-        <v>6098</v>
+        <v>5194</v>
       </c>
       <c r="Q23" s="1">
-        <v>768804</v>
+        <v>697620</v>
       </c>
       <c r="R23" s="2">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="S23" s="1" t="s">
         <v>166</v>
@@ -2668,13 +2668,13 @@
         <v>3403556</v>
       </c>
       <c r="P24" s="1">
-        <v>14861</v>
+        <v>14297</v>
       </c>
       <c r="Q24" s="1">
-        <v>900883</v>
+        <v>872174</v>
       </c>
       <c r="R24" s="2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="S24" s="1" t="s">
         <v>167</v>
@@ -2727,13 +2727,13 @@
         <v>3153302</v>
       </c>
       <c r="P25" s="1">
-        <v>2730</v>
+        <v>2552</v>
       </c>
       <c r="Q25" s="1">
-        <v>509718</v>
+        <v>479332</v>
       </c>
       <c r="R25" s="2">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="S25" s="1" t="s">
         <v>168</v>
@@ -2786,13 +2786,13 @@
         <v>2901328</v>
       </c>
       <c r="P26" s="1">
-        <v>11285</v>
+        <v>10910</v>
       </c>
       <c r="Q26" s="1">
-        <v>1029298</v>
+        <v>985591</v>
       </c>
       <c r="R26" s="2">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="S26" s="1" t="s">
         <v>169</v>
@@ -2845,10 +2845,10 @@
         <v>2481407</v>
       </c>
       <c r="P27" s="1">
-        <v>7086</v>
+        <v>6904</v>
       </c>
       <c r="Q27" s="1">
-        <v>658468</v>
+        <v>641183</v>
       </c>
       <c r="R27" s="2">
         <v>1.5</v>
@@ -2904,13 +2904,13 @@
         <v>2373975</v>
       </c>
       <c r="P28" s="1">
-        <v>6009</v>
+        <v>5461</v>
       </c>
       <c r="Q28" s="1">
-        <v>495653</v>
+        <v>433023</v>
       </c>
       <c r="R28" s="2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="S28" s="1" t="s">
         <v>171</v>
@@ -2963,13 +2963,13 @@
         <v>2127393</v>
       </c>
       <c r="P29" s="1">
-        <v>5943</v>
+        <v>5439</v>
       </c>
       <c r="Q29" s="1">
-        <v>459278</v>
+        <v>408169</v>
       </c>
       <c r="R29" s="2">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="S29" s="1" t="s">
         <v>172</v>
@@ -3022,13 +3022,13 @@
         <v>2051386</v>
       </c>
       <c r="P30" s="1">
-        <v>5862</v>
+        <v>5479</v>
       </c>
       <c r="Q30" s="1">
-        <v>633268</v>
+        <v>581868</v>
       </c>
       <c r="R30" s="2">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="S30" s="1" t="s">
         <v>173</v>
@@ -3081,10 +3081,10 @@
         <v>1996475</v>
       </c>
       <c r="P31" s="1">
-        <v>3224</v>
+        <v>3311</v>
       </c>
       <c r="Q31" s="1">
-        <v>537945</v>
+        <v>536163</v>
       </c>
       <c r="R31" s="2">
         <v>1.6</v>
@@ -3140,13 +3140,13 @@
         <v>1992220</v>
       </c>
       <c r="P32" s="1">
-        <v>4013</v>
+        <v>3699</v>
       </c>
       <c r="Q32" s="1">
-        <v>637402</v>
+        <v>601826</v>
       </c>
       <c r="R32" s="2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="S32" s="1" t="s">
         <v>175</v>
@@ -3199,13 +3199,13 @@
         <v>1952923</v>
       </c>
       <c r="P33" s="1">
-        <v>2225</v>
+        <v>1607</v>
       </c>
       <c r="Q33" s="1">
-        <v>252307</v>
+        <v>185280</v>
       </c>
       <c r="R33" s="2">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
       <c r="S33" s="1" t="s">
         <v>176</v>
@@ -3258,13 +3258,13 @@
         <v>1830717</v>
       </c>
       <c r="P34" s="1">
-        <v>182</v>
+        <v>161</v>
       </c>
       <c r="Q34" s="1">
-        <v>38277</v>
+        <v>34284</v>
       </c>
       <c r="R34" s="2">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="S34" s="1" t="s">
         <v>177</v>
@@ -3317,13 +3317,13 @@
         <v>1729934</v>
       </c>
       <c r="P35" s="1">
-        <v>4959</v>
+        <v>4880</v>
       </c>
       <c r="Q35" s="1">
-        <v>985941</v>
+        <v>956119</v>
       </c>
       <c r="R35" s="2">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="S35" s="1" t="s">
         <v>178</v>
@@ -3376,10 +3376,10 @@
         <v>1719805</v>
       </c>
       <c r="P36" s="1">
-        <v>10934</v>
+        <v>10208</v>
       </c>
       <c r="Q36" s="1">
-        <v>323928</v>
+        <v>283499</v>
       </c>
       <c r="R36" s="2">
         <v>0.8</v>
@@ -3435,13 +3435,13 @@
         <v>1717791</v>
       </c>
       <c r="P37" s="1">
-        <v>8101</v>
+        <v>6740</v>
       </c>
       <c r="Q37" s="1">
-        <v>205375</v>
+        <v>175784</v>
       </c>
       <c r="R37" s="2">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="S37" s="1" t="s">
         <v>54</v>
@@ -3494,13 +3494,13 @@
         <v>1633719</v>
       </c>
       <c r="P38" s="1">
-        <v>7279</v>
+        <v>6928</v>
       </c>
       <c r="Q38" s="1">
-        <v>332080</v>
+        <v>318090</v>
       </c>
       <c r="R38" s="2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="S38" s="1" t="s">
         <v>179</v>
@@ -3553,10 +3553,10 @@
         <v>1613859</v>
       </c>
       <c r="P39" s="1">
-        <v>6022</v>
+        <v>6000</v>
       </c>
       <c r="Q39" s="1">
-        <v>746454</v>
+        <v>743384</v>
       </c>
       <c r="R39" s="2">
         <v>2.4</v>
@@ -3612,13 +3612,13 @@
         <v>1548859</v>
       </c>
       <c r="P40" s="1">
-        <v>1620</v>
+        <v>1438</v>
       </c>
       <c r="Q40" s="1">
-        <v>424966</v>
+        <v>374317</v>
       </c>
       <c r="R40" s="2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="S40" s="1" t="s">
         <v>57</v>
@@ -3671,13 +3671,13 @@
         <v>1536754</v>
       </c>
       <c r="P41" s="1">
-        <v>1647</v>
+        <v>1395</v>
       </c>
       <c r="Q41" s="1">
-        <v>491474</v>
+        <v>411284</v>
       </c>
       <c r="R41" s="2">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="S41" s="1" t="s">
         <v>181</v>
@@ -3730,13 +3730,13 @@
         <v>1502872</v>
       </c>
       <c r="P42" s="1">
-        <v>1217</v>
+        <v>1084</v>
       </c>
       <c r="Q42" s="1">
-        <v>246815</v>
+        <v>209801</v>
       </c>
       <c r="R42" s="2">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="S42" s="1" t="s">
         <v>182</v>
@@ -3789,10 +3789,10 @@
         <v>1414849</v>
       </c>
       <c r="P43" s="1">
-        <v>9920</v>
+        <v>9391</v>
       </c>
       <c r="Q43" s="1">
-        <v>309308</v>
+        <v>275777</v>
       </c>
       <c r="R43" s="2">
         <v>0.8</v>
@@ -3848,13 +3848,13 @@
         <v>1365547</v>
       </c>
       <c r="P44" s="1">
-        <v>3112</v>
+        <v>2932</v>
       </c>
       <c r="Q44" s="1">
-        <v>706473</v>
+        <v>658564</v>
       </c>
       <c r="R44" s="2">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="S44" s="1" t="s">
         <v>184</v>
@@ -3907,10 +3907,10 @@
         <v>1258947</v>
       </c>
       <c r="P45" s="1">
-        <v>12000</v>
+        <v>11860</v>
       </c>
       <c r="Q45" s="1">
-        <v>374813</v>
+        <v>368280</v>
       </c>
       <c r="R45" s="2">
         <v>1.6</v>
@@ -3966,13 +3966,13 @@
         <v>1222686</v>
       </c>
       <c r="P46" s="1">
-        <v>5134</v>
+        <v>4836</v>
       </c>
       <c r="Q46" s="1">
-        <v>224587</v>
+        <v>211227</v>
       </c>
       <c r="R46" s="2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="S46" s="1" t="s">
         <v>186</v>
@@ -4025,13 +4025,13 @@
         <v>1200781</v>
       </c>
       <c r="P47" s="1">
-        <v>11440</v>
+        <v>9660</v>
       </c>
       <c r="Q47" s="1">
-        <v>366010</v>
+        <v>323964</v>
       </c>
       <c r="R47" s="2">
-        <v>2</v>
+        <v>1.7</v>
       </c>
       <c r="S47" s="1" t="s">
         <v>187</v>
@@ -4084,10 +4084,10 @@
         <v>1168782</v>
       </c>
       <c r="P48" s="1">
-        <v>4195</v>
+        <v>4165</v>
       </c>
       <c r="Q48" s="1">
-        <v>429023</v>
+        <v>425752</v>
       </c>
       <c r="R48" s="2">
         <v>2</v>
@@ -4202,10 +4202,10 @@
         <v>1053912</v>
       </c>
       <c r="P50" s="1">
-        <v>2556</v>
+        <v>2537</v>
       </c>
       <c r="Q50" s="1">
-        <v>297945</v>
+        <v>296371</v>
       </c>
       <c r="R50" s="2">
         <v>1.4</v>
@@ -4261,10 +4261,10 @@
         <v>1050243</v>
       </c>
       <c r="P51" s="1">
-        <v>1328</v>
+        <v>1275</v>
       </c>
       <c r="Q51" s="1">
-        <v>451461</v>
+        <v>431675</v>
       </c>
       <c r="R51" s="2">
         <v>0.8</v>
@@ -4320,13 +4320,13 @@
         <v>962277</v>
       </c>
       <c r="P52" s="1">
-        <v>6250</v>
+        <v>6065</v>
       </c>
       <c r="Q52" s="1">
-        <v>719335</v>
+        <v>687010</v>
       </c>
       <c r="R52" s="2">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="S52" s="1" t="s">
         <v>192</v>
@@ -4379,13 +4379,13 @@
         <v>938957</v>
       </c>
       <c r="P53" s="1">
-        <v>2116</v>
+        <v>1761</v>
       </c>
       <c r="Q53" s="1">
-        <v>102159</v>
+        <v>75983</v>
       </c>
       <c r="R53" s="2">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="S53" s="1" t="s">
         <v>193</v>
@@ -4438,10 +4438,10 @@
         <v>917414</v>
       </c>
       <c r="P54" s="1">
-        <v>1237</v>
+        <v>1221</v>
       </c>
       <c r="Q54" s="1">
-        <v>182947</v>
+        <v>180051</v>
       </c>
       <c r="R54" s="2">
         <v>1.1</v>
@@ -4497,13 +4497,13 @@
         <v>869605</v>
       </c>
       <c r="P55" s="1">
-        <v>1201</v>
+        <v>1050</v>
       </c>
       <c r="Q55" s="1">
-        <v>364427</v>
+        <v>314412</v>
       </c>
       <c r="R55" s="2">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="S55" s="1" t="s">
         <v>195</v>
@@ -4556,13 +4556,13 @@
         <v>865930</v>
       </c>
       <c r="P56" s="1">
-        <v>1542</v>
+        <v>1500</v>
       </c>
       <c r="Q56" s="1">
-        <v>332104</v>
+        <v>318152</v>
       </c>
       <c r="R56" s="2">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="S56" s="1" t="s">
         <v>196</v>
@@ -4615,10 +4615,10 @@
         <v>795798</v>
       </c>
       <c r="P57" s="1">
-        <v>880</v>
+        <v>889</v>
       </c>
       <c r="Q57" s="1">
-        <v>302103</v>
+        <v>300454</v>
       </c>
       <c r="R57" s="2">
         <v>1.6</v>
@@ -4674,10 +4674,10 @@
         <v>725876</v>
       </c>
       <c r="P58" s="1">
-        <v>9538</v>
+        <v>9399</v>
       </c>
       <c r="Q58" s="1">
-        <v>505640</v>
+        <v>499040</v>
       </c>
       <c r="R58" s="2">
         <v>4.2</v>
@@ -4733,13 +4733,13 @@
         <v>705719</v>
       </c>
       <c r="P59" s="1">
-        <v>5139</v>
+        <v>4839</v>
       </c>
       <c r="Q59" s="1">
-        <v>365301</v>
+        <v>342558</v>
       </c>
       <c r="R59" s="2">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="S59" s="1" t="s">
         <v>199</v>
@@ -4792,10 +4792,10 @@
         <v>698835</v>
       </c>
       <c r="P60" s="1">
-        <v>1902</v>
+        <v>1881</v>
       </c>
       <c r="Q60" s="1">
-        <v>151898</v>
+        <v>150430</v>
       </c>
       <c r="R60" s="2">
         <v>1.3</v>
@@ -4851,13 +4851,13 @@
         <v>587724</v>
       </c>
       <c r="P61" s="1">
-        <v>4372</v>
+        <v>2863</v>
       </c>
       <c r="Q61" s="1">
-        <v>114338</v>
+        <v>81353</v>
       </c>
       <c r="R61" s="2">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="S61" s="1" t="s">
         <v>201</v>
@@ -4969,10 +4969,10 @@
         <v>576776</v>
       </c>
       <c r="P63" s="1">
-        <v>1693</v>
+        <v>1687</v>
       </c>
       <c r="Q63" s="1">
-        <v>105850</v>
+        <v>104280</v>
       </c>
       <c r="R63" s="2">
         <v>1.2</v>
@@ -5028,13 +5028,13 @@
         <v>569994</v>
       </c>
       <c r="P64" s="1">
-        <v>1187</v>
+        <v>1126</v>
       </c>
       <c r="Q64" s="1">
-        <v>284460</v>
+        <v>279014</v>
       </c>
       <c r="R64" s="2">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="S64" s="1" t="s">
         <v>203</v>
@@ -5087,13 +5087,13 @@
         <v>543885</v>
       </c>
       <c r="P65" s="1">
-        <v>606</v>
+        <v>574</v>
       </c>
       <c r="Q65" s="1">
-        <v>100035</v>
+        <v>93006</v>
       </c>
       <c r="R65" s="2">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="S65" s="1" t="s">
         <v>204</v>
@@ -5146,13 +5146,13 @@
         <v>525089</v>
       </c>
       <c r="P66" s="1">
-        <v>823</v>
+        <v>807</v>
       </c>
       <c r="Q66" s="1">
-        <v>170585</v>
+        <v>160586</v>
       </c>
       <c r="R66" s="2">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="S66" s="1" t="s">
         <v>205</v>
@@ -5205,13 +5205,13 @@
         <v>506044</v>
       </c>
       <c r="P67" s="1">
-        <v>17552</v>
+        <v>17344</v>
       </c>
       <c r="Q67" s="1">
-        <v>847060</v>
+        <v>845962</v>
       </c>
       <c r="R67" s="2">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="S67" s="1" t="s">
         <v>206</v>
@@ -5264,13 +5264,13 @@
         <v>503475</v>
       </c>
       <c r="P68" s="1">
-        <v>4729</v>
+        <v>3691</v>
       </c>
       <c r="Q68" s="1">
-        <v>590344</v>
+        <v>424583</v>
       </c>
       <c r="R68" s="2">
-        <v>5.1</v>
+        <v>4</v>
       </c>
       <c r="S68" s="1" t="s">
         <v>207</v>
@@ -5323,10 +5323,10 @@
         <v>494215</v>
       </c>
       <c r="P69" s="1">
-        <v>2169</v>
+        <v>2182</v>
       </c>
       <c r="Q69" s="1">
-        <v>82913</v>
+        <v>60487</v>
       </c>
       <c r="R69" s="2">
         <v>0.7</v>
@@ -5382,13 +5382,13 @@
         <v>481799</v>
       </c>
       <c r="P70" s="1">
-        <v>2087</v>
+        <v>1927</v>
       </c>
       <c r="Q70" s="1">
-        <v>135680</v>
+        <v>126025</v>
       </c>
       <c r="R70" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="S70" s="1" t="s">
         <v>208</v>
@@ -5441,13 +5441,13 @@
         <v>446545</v>
       </c>
       <c r="P71" s="1">
-        <v>2700</v>
+        <v>2379</v>
       </c>
       <c r="Q71" s="1">
-        <v>228614</v>
+        <v>204901</v>
       </c>
       <c r="R71" s="2">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="S71" s="1" t="s">
         <v>209</v>
@@ -5500,13 +5500,13 @@
         <v>443725</v>
       </c>
       <c r="P72" s="1">
-        <v>926</v>
+        <v>866</v>
       </c>
       <c r="Q72" s="1">
-        <v>84293</v>
+        <v>80986</v>
       </c>
       <c r="R72" s="2">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="S72" s="1" t="s">
         <v>210</v>
@@ -5559,10 +5559,10 @@
         <v>419678</v>
       </c>
       <c r="P73" s="1">
-        <v>3336</v>
+        <v>3280</v>
       </c>
       <c r="Q73" s="1">
-        <v>328466</v>
+        <v>315608</v>
       </c>
       <c r="R73" s="2">
         <v>2.2</v>
@@ -5618,13 +5618,13 @@
         <v>416146</v>
       </c>
       <c r="P74" s="1">
-        <v>552</v>
+        <v>526</v>
       </c>
       <c r="Q74" s="1">
-        <v>325689</v>
+        <v>321039</v>
       </c>
       <c r="R74" s="2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="S74" s="1" t="s">
         <v>212</v>
@@ -5677,13 +5677,13 @@
         <v>399232</v>
       </c>
       <c r="P75" s="1">
-        <v>3056</v>
+        <v>3386</v>
       </c>
       <c r="Q75" s="1">
-        <v>145900</v>
+        <v>145090</v>
       </c>
       <c r="R75" s="2">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
       <c r="S75" s="1" t="s">
         <v>213</v>
@@ -5736,13 +5736,13 @@
         <v>371222</v>
       </c>
       <c r="P76" s="1">
-        <v>3560</v>
+        <v>3480</v>
       </c>
       <c r="Q76" s="1">
-        <v>542018</v>
+        <v>533698</v>
       </c>
       <c r="R76" s="2">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
       <c r="S76" s="1" t="s">
         <v>214</v>
@@ -5795,13 +5795,13 @@
         <v>367850</v>
       </c>
       <c r="P77" s="1">
-        <v>1618</v>
+        <v>1591</v>
       </c>
       <c r="Q77" s="1">
-        <v>147283</v>
+        <v>142194</v>
       </c>
       <c r="R77" s="2">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="S77" s="1" t="s">
         <v>215</v>
@@ -5854,13 +5854,13 @@
         <v>363780</v>
       </c>
       <c r="P78" s="1">
-        <v>3293</v>
+        <v>3243</v>
       </c>
       <c r="Q78" s="1">
-        <v>365008</v>
+        <v>360614</v>
       </c>
       <c r="R78" s="2">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="S78" s="1" t="s">
         <v>216</v>
@@ -5913,10 +5913,10 @@
         <v>356405</v>
       </c>
       <c r="P79" s="1">
-        <v>975</v>
+        <v>980</v>
       </c>
       <c r="Q79" s="1">
-        <v>85170</v>
+        <v>85098</v>
       </c>
       <c r="R79" s="2">
         <v>1.5</v>
@@ -5972,10 +5972,10 @@
         <v>353335</v>
       </c>
       <c r="P80" s="1">
-        <v>1598</v>
+        <v>1586</v>
       </c>
       <c r="Q80" s="1">
-        <v>165988</v>
+        <v>164614</v>
       </c>
       <c r="R80" s="2">
         <v>2.7</v>
@@ -6031,13 +6031,13 @@
         <v>335048</v>
       </c>
       <c r="P81" s="1">
-        <v>1717</v>
+        <v>1589</v>
       </c>
       <c r="Q81" s="1">
-        <v>155882</v>
+        <v>143454</v>
       </c>
       <c r="R81" s="2">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="S81" s="1" t="s">
         <v>219</v>
@@ -6090,10 +6090,10 @@
         <v>312069</v>
       </c>
       <c r="P82" s="1">
-        <v>1887</v>
+        <v>1805</v>
       </c>
       <c r="Q82" s="1">
-        <v>115063</v>
+        <v>112586</v>
       </c>
       <c r="R82" s="2">
         <v>1</v>
@@ -6149,10 +6149,10 @@
         <v>306511</v>
       </c>
       <c r="P83" s="1">
-        <v>887</v>
+        <v>852</v>
       </c>
       <c r="Q83" s="1">
-        <v>82365</v>
+        <v>77956</v>
       </c>
       <c r="R83" s="2">
         <v>1.2</v>
@@ -6208,13 +6208,13 @@
         <v>306374</v>
       </c>
       <c r="P84" s="1">
-        <v>956</v>
+        <v>927</v>
       </c>
       <c r="Q84" s="1">
-        <v>95158</v>
+        <v>92476</v>
       </c>
       <c r="R84" s="2">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="S84" s="1" t="s">
         <v>222</v>
@@ -6267,10 +6267,10 @@
         <v>303328</v>
       </c>
       <c r="P85" s="1">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="Q85" s="1">
-        <v>6152</v>
+        <v>6000</v>
       </c>
       <c r="R85" s="2">
         <v>0.1</v>
@@ -6326,7 +6326,7 @@
         <v>287372</v>
       </c>
       <c r="P86" s="1">
-        <v>1314</v>
+        <v>1324</v>
       </c>
       <c r="Q86" s="1">
         <v>182207</v>
@@ -6385,13 +6385,13 @@
         <v>258797</v>
       </c>
       <c r="P87" s="1">
-        <v>871</v>
+        <v>751</v>
       </c>
       <c r="Q87" s="1">
-        <v>62770</v>
+        <v>53938</v>
       </c>
       <c r="R87" s="2">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="S87" s="1" t="s">
         <v>225</v>
@@ -6444,13 +6444,13 @@
         <v>257112</v>
       </c>
       <c r="P88" s="1">
-        <v>623</v>
+        <v>374</v>
       </c>
       <c r="Q88" s="1">
-        <v>98854</v>
+        <v>69212</v>
       </c>
       <c r="R88" s="2">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
       <c r="S88" s="1" t="s">
         <v>226</v>
@@ -6503,10 +6503,10 @@
         <v>247853</v>
       </c>
       <c r="P89" s="1">
-        <v>5680</v>
+        <v>5678</v>
       </c>
       <c r="Q89" s="1">
-        <v>824972</v>
+        <v>824852</v>
       </c>
       <c r="R89" s="2">
         <v>11.4</v>
@@ -6562,13 +6562,13 @@
         <v>247507</v>
       </c>
       <c r="P90" s="1">
-        <v>603</v>
+        <v>610</v>
       </c>
       <c r="Q90" s="1">
-        <v>102296</v>
+        <v>101210</v>
       </c>
       <c r="R90" s="2">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
       <c r="S90" s="1" t="s">
         <v>228</v>
@@ -6621,13 +6621,13 @@
         <v>232232</v>
       </c>
       <c r="P91" s="1">
-        <v>91</v>
+        <v>34</v>
       </c>
       <c r="Q91" s="1">
-        <v>18737</v>
+        <v>9155</v>
       </c>
       <c r="R91" s="2">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="S91" s="1" t="s">
         <v>229</v>
@@ -6680,13 +6680,13 @@
         <v>228869</v>
       </c>
       <c r="P92" s="1">
-        <v>959</v>
+        <v>834</v>
       </c>
       <c r="Q92" s="1">
-        <v>61533</v>
+        <v>53338</v>
       </c>
       <c r="R92" s="2">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="S92" s="1" t="s">
         <v>230</v>
@@ -6739,13 +6739,13 @@
         <v>222516</v>
       </c>
       <c r="P93" s="1">
-        <v>4873</v>
+        <v>4748</v>
       </c>
       <c r="Q93" s="1">
-        <v>582922</v>
+        <v>565737</v>
       </c>
       <c r="R93" s="2">
-        <v>12</v>
+        <v>11.7</v>
       </c>
       <c r="S93" s="1" t="s">
         <v>231</v>
@@ -6798,10 +6798,10 @@
         <v>209820</v>
       </c>
       <c r="P94" s="1">
-        <v>3500</v>
+        <v>3478</v>
       </c>
       <c r="Q94" s="1">
-        <v>189934</v>
+        <v>188378</v>
       </c>
       <c r="R94" s="2">
         <v>5.7</v>
@@ -6857,10 +6857,10 @@
         <v>205272</v>
       </c>
       <c r="P95" s="1">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="Q95" s="1">
-        <v>123683</v>
+        <v>122694</v>
       </c>
       <c r="R95" s="2">
         <v>2.7</v>
@@ -6916,10 +6916,10 @@
         <v>188616</v>
       </c>
       <c r="P96" s="1">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="Q96" s="1">
-        <v>58593</v>
+        <v>58343</v>
       </c>
       <c r="R96" s="2">
         <v>1.8</v>
@@ -6975,13 +6975,13 @@
         <v>181446</v>
       </c>
       <c r="P97" s="1">
-        <v>1816</v>
+        <v>1773</v>
       </c>
       <c r="Q97" s="1">
-        <v>117499</v>
+        <v>112606</v>
       </c>
       <c r="R97" s="2">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="S97" s="1" t="s">
         <v>235</v>
@@ -7093,13 +7093,13 @@
         <v>166081</v>
       </c>
       <c r="P99" s="1">
-        <v>1304</v>
+        <v>1276</v>
       </c>
       <c r="Q99" s="1">
-        <v>116369</v>
+        <v>111764</v>
       </c>
       <c r="R99" s="2">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="S99" s="1" t="s">
         <v>237</v>
@@ -7152,10 +7152,10 @@
         <v>165708</v>
       </c>
       <c r="P100" s="1">
-        <v>526</v>
+        <v>505</v>
       </c>
       <c r="Q100" s="1">
-        <v>26563</v>
+        <v>25766</v>
       </c>
       <c r="R100" s="2">
         <v>0.9</v>
@@ -7211,13 +7211,13 @@
         <v>162658</v>
       </c>
       <c r="P101" s="1">
-        <v>2785</v>
+        <v>2464</v>
       </c>
       <c r="Q101" s="1">
-        <v>84261</v>
+        <v>78163</v>
       </c>
       <c r="R101" s="2">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="S101" s="1" t="s">
         <v>239</v>
@@ -7270,10 +7270,10 @@
         <v>160758</v>
       </c>
       <c r="P102" s="1">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="Q102" s="1">
-        <v>119460</v>
+        <v>119198</v>
       </c>
       <c r="R102" s="2">
         <v>4.4</v>
@@ -7329,13 +7329,13 @@
         <v>155919</v>
       </c>
       <c r="P103" s="1">
-        <v>1332</v>
+        <v>1234</v>
       </c>
       <c r="Q103" s="1">
-        <v>56555</v>
+        <v>52432</v>
       </c>
       <c r="R103" s="2">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="S103" s="1" t="s">
         <v>241</v>
@@ -7388,10 +7388,10 @@
         <v>145054</v>
       </c>
       <c r="P104" s="1">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="Q104" s="1">
-        <v>120437</v>
+        <v>118606</v>
       </c>
       <c r="R104" s="2">
         <v>3.3</v>
@@ -7447,10 +7447,10 @@
         <v>125380</v>
       </c>
       <c r="P105" s="1">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="Q105" s="1">
-        <v>37981</v>
+        <v>36241</v>
       </c>
       <c r="R105" s="2">
         <v>1.7</v>
@@ -7506,10 +7506,10 @@
         <v>119439</v>
       </c>
       <c r="P106" s="1">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="Q106" s="1">
-        <v>36824</v>
+        <v>36775</v>
       </c>
       <c r="R106" s="2">
         <v>1.8</v>
@@ -7624,13 +7624,13 @@
         <v>108899</v>
       </c>
       <c r="P108" s="1">
-        <v>462</v>
+        <v>416</v>
       </c>
       <c r="Q108" s="1">
-        <v>23593</v>
+        <v>21236</v>
       </c>
       <c r="R108" s="2">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="S108" s="1" t="s">
         <v>246</v>
@@ -7683,13 +7683,13 @@
         <v>85756</v>
       </c>
       <c r="P109" s="1">
-        <v>192</v>
+        <v>79</v>
       </c>
       <c r="Q109" s="1">
-        <v>17455</v>
+        <v>5286</v>
       </c>
       <c r="R109" s="2">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="S109" s="1" t="s">
         <v>247</v>
@@ -7742,10 +7742,10 @@
         <v>77595</v>
       </c>
       <c r="P110" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q110" s="1">
-        <v>295</v>
+        <v>258</v>
       </c>
       <c r="R110" s="2">
         <v>0</v>
@@ -7860,10 +7860,10 @@
         <v>70476</v>
       </c>
       <c r="P112" s="1">
-        <v>442</v>
+        <v>422</v>
       </c>
       <c r="Q112" s="1">
-        <v>13614</v>
+        <v>13014</v>
       </c>
       <c r="R112" s="2">
         <v>1.1</v>
@@ -7919,13 +7919,13 @@
         <v>65173</v>
       </c>
       <c r="P113" s="1">
-        <v>387</v>
+        <v>261</v>
       </c>
       <c r="Q113" s="1">
-        <v>26053</v>
+        <v>19109</v>
       </c>
       <c r="R113" s="2">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
       <c r="S113" s="1" t="s">
         <v>251</v>
@@ -7978,13 +7978,13 @@
         <v>61440</v>
       </c>
       <c r="P114" s="1">
-        <v>258</v>
+        <v>166</v>
       </c>
       <c r="Q114" s="1">
-        <v>10610</v>
+        <v>7950</v>
       </c>
       <c r="R114" s="2">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="S114" s="1" t="s">
         <v>252</v>
@@ -8155,13 +8155,13 @@
         <v>36954</v>
       </c>
       <c r="P117" s="1">
-        <v>2263</v>
+        <v>2186</v>
       </c>
       <c r="Q117" s="1">
-        <v>67176</v>
+        <v>64866</v>
       </c>
       <c r="R117" s="2">
-        <v>11</v>
+        <v>10.6</v>
       </c>
       <c r="S117" s="1" t="s">
         <v>255</v>
@@ -8214,13 +8214,13 @@
         <v>34286</v>
       </c>
       <c r="P118" s="1">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Q118" s="1">
-        <v>33886</v>
+        <v>33271</v>
       </c>
       <c r="R118" s="2">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="S118" s="1" t="s">
         <v>256</v>
@@ -8273,10 +8273,10 @@
         <v>30897</v>
       </c>
       <c r="P119" s="1">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="Q119" s="1">
-        <v>10473</v>
+        <v>10353</v>
       </c>
       <c r="R119" s="2">
         <v>0</v>
@@ -8332,10 +8332,10 @@
         <v>25268</v>
       </c>
       <c r="P120" s="1">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q120" s="1">
-        <v>9855</v>
+        <v>9791</v>
       </c>
       <c r="R120" s="2">
         <v>2.5</v>
@@ -8450,13 +8450,13 @@
         <v>2439</v>
       </c>
       <c r="P122" s="1">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="Q122" s="1">
-        <v>2089</v>
+        <v>1347</v>
       </c>
       <c r="R122" s="2">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
       <c r="S122" s="1" t="s">
         <v>260</v>
@@ -8568,13 +8568,13 @@
         <v>94</v>
       </c>
       <c r="P124" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q124" s="1">
-        <v>1201</v>
+        <v>1030</v>
       </c>
       <c r="R124" s="2">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="S124" s="1" t="s">
         <v>262</v>
@@ -8627,10 +8627,10 @@
         <v>0</v>
       </c>
       <c r="P125" s="1">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="Q125" s="1">
-        <v>1159</v>
+        <v>1102</v>
       </c>
       <c r="S125" s="1" t="s">
         <v>263</v>
@@ -8683,10 +8683,10 @@
         <v>0</v>
       </c>
       <c r="P126" s="1">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="Q126" s="1">
-        <v>556</v>
+        <v>40</v>
       </c>
       <c r="S126" s="1" t="s">
         <v>264</v>
@@ -8882,13 +8882,13 @@
         <v>54255889</v>
       </c>
       <c r="Q2" s="1">
-        <v>303751</v>
+        <v>282991</v>
       </c>
       <c r="R2" s="1">
-        <v>25252505</v>
+        <v>23708597</v>
       </c>
       <c r="S2" s="2">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -8941,13 +8941,13 @@
         <v>45524507</v>
       </c>
       <c r="Q3" s="1">
-        <v>136428</v>
+        <v>129700</v>
       </c>
       <c r="R3" s="1">
-        <v>24486238</v>
+        <v>23338272</v>
       </c>
       <c r="S3" s="2">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -9000,10 +9000,10 @@
         <v>20240180</v>
       </c>
       <c r="Q4" s="1">
-        <v>12837</v>
+        <v>12140</v>
       </c>
       <c r="R4" s="1">
-        <v>1223754</v>
+        <v>1137858</v>
       </c>
       <c r="S4" s="2">
         <v>0.2</v>
@@ -9059,10 +9059,10 @@
         <v>15679727</v>
       </c>
       <c r="Q5" s="1">
-        <v>68554</v>
+        <v>67373</v>
       </c>
       <c r="R5" s="1">
-        <v>2828335</v>
+        <v>2742626</v>
       </c>
       <c r="S5" s="2">
         <v>1.1</v>
@@ -9118,13 +9118,13 @@
         <v>14141465</v>
       </c>
       <c r="Q6" s="1">
-        <v>23610</v>
+        <v>21408</v>
       </c>
       <c r="R6" s="1">
-        <v>6500477</v>
+        <v>5847457</v>
       </c>
       <c r="S6" s="2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="7" spans="1:19">
@@ -9177,10 +9177,10 @@
         <v>12011598</v>
       </c>
       <c r="Q7" s="1">
-        <v>14147</v>
+        <v>13679</v>
       </c>
       <c r="R7" s="1">
-        <v>3552844</v>
+        <v>3446164</v>
       </c>
       <c r="S7" s="2">
         <v>1.7</v>
@@ -9236,10 +9236,10 @@
         <v>9717919</v>
       </c>
       <c r="Q8" s="1">
-        <v>44641</v>
+        <v>42622</v>
       </c>
       <c r="R8" s="1">
-        <v>2528189</v>
+        <v>2339330</v>
       </c>
       <c r="S8" s="2">
         <v>1</v>
@@ -9295,10 +9295,10 @@
         <v>9534356</v>
       </c>
       <c r="Q9" s="1">
-        <v>47124</v>
+        <v>45592</v>
       </c>
       <c r="R9" s="1">
-        <v>1829193</v>
+        <v>1760405</v>
       </c>
       <c r="S9" s="2">
         <v>1.1</v>
@@ -9354,10 +9354,10 @@
         <v>9145683</v>
       </c>
       <c r="Q10" s="1">
-        <v>66050</v>
+        <v>64494</v>
       </c>
       <c r="R10" s="1">
-        <v>2043610</v>
+        <v>1867763</v>
       </c>
       <c r="S10" s="2">
         <v>1.2</v>
@@ -9413,13 +9413,13 @@
         <v>7582485</v>
       </c>
       <c r="Q11" s="1">
-        <v>22259</v>
+        <v>21256</v>
       </c>
       <c r="R11" s="1">
-        <v>3347660</v>
+        <v>3199031</v>
       </c>
       <c r="S11" s="2">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="12" spans="1:19">
@@ -9472,13 +9472,13 @@
         <v>7525182</v>
       </c>
       <c r="Q12" s="1">
-        <v>41334</v>
+        <v>39224</v>
       </c>
       <c r="R12" s="1">
-        <v>3839063</v>
+        <v>3616851</v>
       </c>
       <c r="S12" s="2">
-        <v>3.1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -9531,10 +9531,10 @@
         <v>7324462</v>
       </c>
       <c r="Q13" s="1">
-        <v>39820</v>
+        <v>38832</v>
       </c>
       <c r="R13" s="1">
-        <v>2851192</v>
+        <v>2748271</v>
       </c>
       <c r="S13" s="2">
         <v>1.3</v>
@@ -9590,10 +9590,10 @@
         <v>5553389</v>
       </c>
       <c r="Q14" s="1">
-        <v>35058</v>
+        <v>33410</v>
       </c>
       <c r="R14" s="1">
-        <v>1330395</v>
+        <v>1255401</v>
       </c>
       <c r="S14" s="2">
         <v>1.3</v>
@@ -9649,13 +9649,13 @@
         <v>5479176</v>
       </c>
       <c r="Q15" s="1">
-        <v>11405</v>
+        <v>10991</v>
       </c>
       <c r="R15" s="1">
-        <v>1524618</v>
+        <v>1453998</v>
       </c>
       <c r="S15" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -9708,10 +9708,10 @@
         <v>4805108</v>
       </c>
       <c r="Q16" s="1">
-        <v>7315</v>
+        <v>6605</v>
       </c>
       <c r="R16" s="1">
-        <v>889693</v>
+        <v>802384</v>
       </c>
       <c r="S16" s="2">
         <v>0.9</v>
@@ -9767,13 +9767,13 @@
         <v>4518071</v>
       </c>
       <c r="Q17" s="1">
-        <v>11325</v>
+        <v>9527</v>
       </c>
       <c r="R17" s="1">
-        <v>511896</v>
+        <v>423606</v>
       </c>
       <c r="S17" s="2">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="18" spans="1:19">
@@ -9826,13 +9826,13 @@
         <v>4334035</v>
       </c>
       <c r="Q18" s="1">
-        <v>6425</v>
+        <v>6054</v>
       </c>
       <c r="R18" s="1">
-        <v>964848</v>
+        <v>920395</v>
       </c>
       <c r="S18" s="2">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -9885,13 +9885,13 @@
         <v>4216981</v>
       </c>
       <c r="Q19" s="1">
-        <v>5763</v>
+        <v>5374</v>
       </c>
       <c r="R19" s="1">
-        <v>926159</v>
+        <v>866785</v>
       </c>
       <c r="S19" s="2">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:19">
@@ -9944,13 +9944,13 @@
         <v>3849754</v>
       </c>
       <c r="Q20" s="1">
-        <v>5384</v>
+        <v>4955</v>
       </c>
       <c r="R20" s="1">
-        <v>604160</v>
+        <v>552635</v>
       </c>
       <c r="S20" s="2">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="21" spans="1:19">
@@ -10003,13 +10003,13 @@
         <v>3564517</v>
       </c>
       <c r="Q21" s="1">
-        <v>9639</v>
+        <v>9202</v>
       </c>
       <c r="R21" s="1">
-        <v>1440432</v>
+        <v>1361837</v>
       </c>
       <c r="S21" s="2">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="22" spans="1:19">
@@ -10062,10 +10062,10 @@
         <v>3485757</v>
       </c>
       <c r="Q22" s="1">
-        <v>12425</v>
+        <v>11994</v>
       </c>
       <c r="R22" s="1">
-        <v>774102</v>
+        <v>743892</v>
       </c>
       <c r="S22" s="2">
         <v>1.3</v>
@@ -10121,13 +10121,13 @@
         <v>3421998</v>
       </c>
       <c r="Q23" s="1">
-        <v>6098</v>
+        <v>5194</v>
       </c>
       <c r="R23" s="1">
-        <v>768804</v>
+        <v>697620</v>
       </c>
       <c r="S23" s="2">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="24" spans="1:19">
@@ -10180,13 +10180,13 @@
         <v>3403556</v>
       </c>
       <c r="Q24" s="1">
-        <v>14861</v>
+        <v>14297</v>
       </c>
       <c r="R24" s="1">
-        <v>900883</v>
+        <v>872174</v>
       </c>
       <c r="S24" s="2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="25" spans="1:19">
@@ -10239,13 +10239,13 @@
         <v>3153302</v>
       </c>
       <c r="Q25" s="1">
-        <v>2730</v>
+        <v>2552</v>
       </c>
       <c r="R25" s="1">
-        <v>509718</v>
+        <v>479332</v>
       </c>
       <c r="S25" s="2">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="26" spans="1:19">
@@ -10298,13 +10298,13 @@
         <v>2901328</v>
       </c>
       <c r="Q26" s="1">
-        <v>11285</v>
+        <v>10910</v>
       </c>
       <c r="R26" s="1">
-        <v>1029298</v>
+        <v>985591</v>
       </c>
       <c r="S26" s="2">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="27" spans="1:19">
@@ -10357,13 +10357,13 @@
         <v>2127393</v>
       </c>
       <c r="Q27" s="1">
-        <v>5943</v>
+        <v>5439</v>
       </c>
       <c r="R27" s="1">
-        <v>459278</v>
+        <v>408169</v>
       </c>
       <c r="S27" s="2">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="28" spans="1:19">
@@ -10416,13 +10416,13 @@
         <v>2051386</v>
       </c>
       <c r="Q28" s="1">
-        <v>5862</v>
+        <v>5479</v>
       </c>
       <c r="R28" s="1">
-        <v>633268</v>
+        <v>581868</v>
       </c>
       <c r="S28" s="2">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="29" spans="1:19">
@@ -10475,10 +10475,10 @@
         <v>1996475</v>
       </c>
       <c r="Q29" s="1">
-        <v>3224</v>
+        <v>3311</v>
       </c>
       <c r="R29" s="1">
-        <v>537945</v>
+        <v>536163</v>
       </c>
       <c r="S29" s="2">
         <v>1.6</v>
@@ -10534,13 +10534,13 @@
         <v>1992220</v>
       </c>
       <c r="Q30" s="1">
-        <v>4013</v>
+        <v>3699</v>
       </c>
       <c r="R30" s="1">
-        <v>637402</v>
+        <v>601826</v>
       </c>
       <c r="S30" s="2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="31" spans="1:19">
@@ -10593,13 +10593,13 @@
         <v>1952923</v>
       </c>
       <c r="Q31" s="1">
-        <v>2225</v>
+        <v>1607</v>
       </c>
       <c r="R31" s="1">
-        <v>252307</v>
+        <v>185280</v>
       </c>
       <c r="S31" s="2">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="32" spans="1:19">
@@ -10652,13 +10652,13 @@
         <v>1830717</v>
       </c>
       <c r="Q32" s="1">
-        <v>182</v>
+        <v>161</v>
       </c>
       <c r="R32" s="1">
-        <v>38277</v>
+        <v>34284</v>
       </c>
       <c r="S32" s="2">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="33" spans="1:19">
@@ -10711,13 +10711,13 @@
         <v>1729934</v>
       </c>
       <c r="Q33" s="1">
-        <v>4959</v>
+        <v>4880</v>
       </c>
       <c r="R33" s="1">
-        <v>985941</v>
+        <v>956119</v>
       </c>
       <c r="S33" s="2">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="34" spans="1:19">
@@ -10770,10 +10770,10 @@
         <v>1719805</v>
       </c>
       <c r="Q34" s="1">
-        <v>10934</v>
+        <v>10208</v>
       </c>
       <c r="R34" s="1">
-        <v>323928</v>
+        <v>283499</v>
       </c>
       <c r="S34" s="2">
         <v>0.8</v>
@@ -10829,13 +10829,13 @@
         <v>1717791</v>
       </c>
       <c r="Q35" s="1">
-        <v>8101</v>
+        <v>6740</v>
       </c>
       <c r="R35" s="1">
-        <v>205375</v>
+        <v>175784</v>
       </c>
       <c r="S35" s="2">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="36" spans="1:19">
@@ -10888,13 +10888,13 @@
         <v>1710906</v>
       </c>
       <c r="Q36" s="1">
-        <v>4463</v>
+        <v>4336</v>
       </c>
       <c r="R36" s="1">
-        <v>432534</v>
+        <v>419804</v>
       </c>
       <c r="S36" s="2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="37" spans="1:19">
@@ -10947,13 +10947,13 @@
         <v>1633719</v>
       </c>
       <c r="Q37" s="1">
-        <v>7279</v>
+        <v>6928</v>
       </c>
       <c r="R37" s="1">
-        <v>332080</v>
+        <v>318090</v>
       </c>
       <c r="S37" s="2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="38" spans="1:19">
@@ -11006,10 +11006,10 @@
         <v>1613859</v>
       </c>
       <c r="Q38" s="1">
-        <v>6022</v>
+        <v>6000</v>
       </c>
       <c r="R38" s="1">
-        <v>746454</v>
+        <v>743384</v>
       </c>
       <c r="S38" s="2">
         <v>2.4</v>
@@ -11065,13 +11065,13 @@
         <v>1548859</v>
       </c>
       <c r="Q39" s="1">
-        <v>1620</v>
+        <v>1438</v>
       </c>
       <c r="R39" s="1">
-        <v>424966</v>
+        <v>374317</v>
       </c>
       <c r="S39" s="2">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="40" spans="1:19">
@@ -11124,13 +11124,13 @@
         <v>1541969</v>
       </c>
       <c r="Q40" s="1">
-        <v>1373</v>
+        <v>928</v>
       </c>
       <c r="R40" s="1">
-        <v>156825</v>
+        <v>105418</v>
       </c>
       <c r="S40" s="2">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="41" spans="1:19">
@@ -11183,13 +11183,13 @@
         <v>1536754</v>
       </c>
       <c r="Q41" s="1">
-        <v>1647</v>
+        <v>1395</v>
       </c>
       <c r="R41" s="1">
-        <v>491474</v>
+        <v>411284</v>
       </c>
       <c r="S41" s="2">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="42" spans="1:19">
@@ -11242,13 +11242,13 @@
         <v>1502872</v>
       </c>
       <c r="Q42" s="1">
-        <v>1217</v>
+        <v>1084</v>
       </c>
       <c r="R42" s="1">
-        <v>246815</v>
+        <v>209801</v>
       </c>
       <c r="S42" s="2">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="43" spans="1:19">
@@ -11301,10 +11301,10 @@
         <v>1414849</v>
       </c>
       <c r="Q43" s="1">
-        <v>9920</v>
+        <v>9391</v>
       </c>
       <c r="R43" s="1">
-        <v>309308</v>
+        <v>275777</v>
       </c>
       <c r="S43" s="2">
         <v>0.8</v>
@@ -11360,13 +11360,13 @@
         <v>1365547</v>
       </c>
       <c r="Q44" s="1">
-        <v>3112</v>
+        <v>2932</v>
       </c>
       <c r="R44" s="1">
-        <v>706473</v>
+        <v>658564</v>
       </c>
       <c r="S44" s="2">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="45" spans="1:19">
@@ -11419,10 +11419,10 @@
         <v>1258947</v>
       </c>
       <c r="Q45" s="1">
-        <v>12000</v>
+        <v>11860</v>
       </c>
       <c r="R45" s="1">
-        <v>374813</v>
+        <v>368280</v>
       </c>
       <c r="S45" s="2">
         <v>1.6</v>
@@ -11478,13 +11478,13 @@
         <v>1222686</v>
       </c>
       <c r="Q46" s="1">
-        <v>5134</v>
+        <v>4836</v>
       </c>
       <c r="R46" s="1">
-        <v>224587</v>
+        <v>211227</v>
       </c>
       <c r="S46" s="2">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="47" spans="1:19">
@@ -11537,13 +11537,13 @@
         <v>1200781</v>
       </c>
       <c r="Q47" s="1">
-        <v>11440</v>
+        <v>9660</v>
       </c>
       <c r="R47" s="1">
-        <v>366010</v>
+        <v>323964</v>
       </c>
       <c r="S47" s="2">
-        <v>2</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="48" spans="1:19">
@@ -11596,10 +11596,10 @@
         <v>1168782</v>
       </c>
       <c r="Q48" s="1">
-        <v>4195</v>
+        <v>4165</v>
       </c>
       <c r="R48" s="1">
-        <v>429023</v>
+        <v>425752</v>
       </c>
       <c r="S48" s="2">
         <v>2</v>
@@ -11714,10 +11714,10 @@
         <v>1053912</v>
       </c>
       <c r="Q50" s="1">
-        <v>2556</v>
+        <v>2537</v>
       </c>
       <c r="R50" s="1">
-        <v>297945</v>
+        <v>296371</v>
       </c>
       <c r="S50" s="2">
         <v>1.4</v>
@@ -11773,13 +11773,13 @@
         <v>962277</v>
       </c>
       <c r="Q51" s="1">
-        <v>6250</v>
+        <v>6065</v>
       </c>
       <c r="R51" s="1">
-        <v>719335</v>
+        <v>687010</v>
       </c>
       <c r="S51" s="2">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="52" spans="1:19">
@@ -11832,13 +11832,13 @@
         <v>938957</v>
       </c>
       <c r="Q52" s="1">
-        <v>2116</v>
+        <v>1761</v>
       </c>
       <c r="R52" s="1">
-        <v>102159</v>
+        <v>75983</v>
       </c>
       <c r="S52" s="2">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="53" spans="1:19">
@@ -11891,10 +11891,10 @@
         <v>917414</v>
       </c>
       <c r="Q53" s="1">
-        <v>1237</v>
+        <v>1221</v>
       </c>
       <c r="R53" s="1">
-        <v>182947</v>
+        <v>180051</v>
       </c>
       <c r="S53" s="2">
         <v>1.1</v>
@@ -11950,13 +11950,13 @@
         <v>869605</v>
       </c>
       <c r="Q54" s="1">
-        <v>1201</v>
+        <v>1050</v>
       </c>
       <c r="R54" s="1">
-        <v>364427</v>
+        <v>314412</v>
       </c>
       <c r="S54" s="2">
-        <v>2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="55" spans="1:19">
@@ -12009,13 +12009,13 @@
         <v>865930</v>
       </c>
       <c r="Q55" s="1">
-        <v>1542</v>
+        <v>1500</v>
       </c>
       <c r="R55" s="1">
-        <v>332104</v>
+        <v>318152</v>
       </c>
       <c r="S55" s="2">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="56" spans="1:19">
@@ -12068,10 +12068,10 @@
         <v>795798</v>
       </c>
       <c r="Q56" s="1">
-        <v>880</v>
+        <v>889</v>
       </c>
       <c r="R56" s="1">
-        <v>302103</v>
+        <v>300454</v>
       </c>
       <c r="S56" s="2">
         <v>1.6</v>
@@ -12127,13 +12127,13 @@
         <v>771123</v>
       </c>
       <c r="Q57" s="1">
-        <v>1128</v>
+        <v>1082</v>
       </c>
       <c r="R57" s="1">
-        <v>444020</v>
+        <v>424549</v>
       </c>
       <c r="S57" s="2">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="58" spans="1:19">
@@ -12186,10 +12186,10 @@
         <v>770501</v>
       </c>
       <c r="Q58" s="1">
-        <v>2623</v>
+        <v>2568</v>
       </c>
       <c r="R58" s="1">
-        <v>225934</v>
+        <v>221379</v>
       </c>
       <c r="S58" s="2">
         <v>1.5</v>
@@ -12245,10 +12245,10 @@
         <v>725876</v>
       </c>
       <c r="Q59" s="1">
-        <v>9538</v>
+        <v>9399</v>
       </c>
       <c r="R59" s="1">
-        <v>505640</v>
+        <v>499040</v>
       </c>
       <c r="S59" s="2">
         <v>4.2</v>
@@ -12304,13 +12304,13 @@
         <v>705719</v>
       </c>
       <c r="Q60" s="1">
-        <v>5139</v>
+        <v>4839</v>
       </c>
       <c r="R60" s="1">
-        <v>365301</v>
+        <v>342558</v>
       </c>
       <c r="S60" s="2">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="61" spans="1:19">
@@ -12363,10 +12363,10 @@
         <v>698835</v>
       </c>
       <c r="Q61" s="1">
-        <v>1902</v>
+        <v>1881</v>
       </c>
       <c r="R61" s="1">
-        <v>151898</v>
+        <v>150430</v>
       </c>
       <c r="S61" s="2">
         <v>1.3</v>
@@ -12422,13 +12422,13 @@
         <v>587724</v>
       </c>
       <c r="Q62" s="1">
-        <v>4372</v>
+        <v>2863</v>
       </c>
       <c r="R62" s="1">
-        <v>114338</v>
+        <v>81353</v>
       </c>
       <c r="S62" s="2">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="63" spans="1:19">
@@ -12540,10 +12540,10 @@
         <v>576776</v>
       </c>
       <c r="Q64" s="1">
-        <v>1693</v>
+        <v>1687</v>
       </c>
       <c r="R64" s="1">
-        <v>105850</v>
+        <v>104280</v>
       </c>
       <c r="S64" s="2">
         <v>1.2</v>
@@ -12599,13 +12599,13 @@
         <v>569994</v>
       </c>
       <c r="Q65" s="1">
-        <v>1187</v>
+        <v>1126</v>
       </c>
       <c r="R65" s="1">
-        <v>284460</v>
+        <v>279014</v>
       </c>
       <c r="S65" s="2">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="66" spans="1:19">
@@ -12658,13 +12658,13 @@
         <v>543885</v>
       </c>
       <c r="Q66" s="1">
-        <v>606</v>
+        <v>574</v>
       </c>
       <c r="R66" s="1">
-        <v>100035</v>
+        <v>93006</v>
       </c>
       <c r="S66" s="2">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="67" spans="1:19">
@@ -12717,13 +12717,13 @@
         <v>525089</v>
       </c>
       <c r="Q67" s="1">
-        <v>823</v>
+        <v>807</v>
       </c>
       <c r="R67" s="1">
-        <v>170585</v>
+        <v>160586</v>
       </c>
       <c r="S67" s="2">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="68" spans="1:19">
@@ -12776,13 +12776,13 @@
         <v>507215</v>
       </c>
       <c r="Q68" s="1">
-        <v>1084</v>
+        <v>999</v>
       </c>
       <c r="R68" s="1">
-        <v>87308</v>
+        <v>78063</v>
       </c>
       <c r="S68" s="2">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="69" spans="1:19">
@@ -12835,13 +12835,13 @@
         <v>506044</v>
       </c>
       <c r="Q69" s="1">
-        <v>17552</v>
+        <v>17344</v>
       </c>
       <c r="R69" s="1">
-        <v>847060</v>
+        <v>845962</v>
       </c>
       <c r="S69" s="2">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="70" spans="1:19">
@@ -12894,13 +12894,13 @@
         <v>503475</v>
       </c>
       <c r="Q70" s="1">
-        <v>4729</v>
+        <v>3691</v>
       </c>
       <c r="R70" s="1">
-        <v>590344</v>
+        <v>424583</v>
       </c>
       <c r="S70" s="2">
-        <v>5.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71" spans="1:19">
@@ -12953,10 +12953,10 @@
         <v>494215</v>
       </c>
       <c r="Q71" s="1">
-        <v>2169</v>
+        <v>2182</v>
       </c>
       <c r="R71" s="1">
-        <v>82913</v>
+        <v>60487</v>
       </c>
       <c r="S71" s="2">
         <v>0.7</v>
@@ -13012,13 +13012,13 @@
         <v>481799</v>
       </c>
       <c r="Q72" s="1">
-        <v>2087</v>
+        <v>1927</v>
       </c>
       <c r="R72" s="1">
-        <v>135680</v>
+        <v>126025</v>
       </c>
       <c r="S72" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="73" spans="1:19">
@@ -13071,13 +13071,13 @@
         <v>446545</v>
       </c>
       <c r="Q73" s="1">
-        <v>2700</v>
+        <v>2379</v>
       </c>
       <c r="R73" s="1">
-        <v>228614</v>
+        <v>204901</v>
       </c>
       <c r="S73" s="2">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="74" spans="1:19">
@@ -13130,13 +13130,13 @@
         <v>443725</v>
       </c>
       <c r="Q74" s="1">
-        <v>926</v>
+        <v>866</v>
       </c>
       <c r="R74" s="1">
-        <v>84293</v>
+        <v>80986</v>
       </c>
       <c r="S74" s="2">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:19">
@@ -13189,10 +13189,10 @@
         <v>419678</v>
       </c>
       <c r="Q75" s="1">
-        <v>3336</v>
+        <v>3280</v>
       </c>
       <c r="R75" s="1">
-        <v>328466</v>
+        <v>315608</v>
       </c>
       <c r="S75" s="2">
         <v>2.2</v>
@@ -13248,13 +13248,13 @@
         <v>416146</v>
       </c>
       <c r="Q76" s="1">
-        <v>552</v>
+        <v>526</v>
       </c>
       <c r="R76" s="1">
-        <v>325689</v>
+        <v>321039</v>
       </c>
       <c r="S76" s="2">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="77" spans="1:19">
@@ -13307,13 +13307,13 @@
         <v>399232</v>
       </c>
       <c r="Q77" s="1">
-        <v>3056</v>
+        <v>3386</v>
       </c>
       <c r="R77" s="1">
-        <v>145900</v>
+        <v>145090</v>
       </c>
       <c r="S77" s="2">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="78" spans="1:19">
@@ -13366,13 +13366,13 @@
         <v>371222</v>
       </c>
       <c r="Q78" s="1">
-        <v>3560</v>
+        <v>3480</v>
       </c>
       <c r="R78" s="1">
-        <v>542018</v>
+        <v>533698</v>
       </c>
       <c r="S78" s="2">
-        <v>6.3</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="79" spans="1:19">
@@ -13425,13 +13425,13 @@
         <v>367850</v>
       </c>
       <c r="Q79" s="1">
-        <v>1618</v>
+        <v>1591</v>
       </c>
       <c r="R79" s="1">
-        <v>147283</v>
+        <v>142194</v>
       </c>
       <c r="S79" s="2">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="80" spans="1:19">
@@ -13484,13 +13484,13 @@
         <v>363780</v>
       </c>
       <c r="Q80" s="1">
-        <v>3293</v>
+        <v>3243</v>
       </c>
       <c r="R80" s="1">
-        <v>365008</v>
+        <v>360614</v>
       </c>
       <c r="S80" s="2">
-        <v>6.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81" spans="1:19">
@@ -13543,10 +13543,10 @@
         <v>356405</v>
       </c>
       <c r="Q81" s="1">
-        <v>975</v>
+        <v>980</v>
       </c>
       <c r="R81" s="1">
-        <v>85170</v>
+        <v>85098</v>
       </c>
       <c r="S81" s="2">
         <v>1.5</v>
@@ -13602,10 +13602,10 @@
         <v>353335</v>
       </c>
       <c r="Q82" s="1">
-        <v>1598</v>
+        <v>1586</v>
       </c>
       <c r="R82" s="1">
-        <v>165988</v>
+        <v>164614</v>
       </c>
       <c r="S82" s="2">
         <v>2.7</v>
@@ -13661,13 +13661,13 @@
         <v>335048</v>
       </c>
       <c r="Q83" s="1">
-        <v>1717</v>
+        <v>1589</v>
       </c>
       <c r="R83" s="1">
-        <v>155882</v>
+        <v>143454</v>
       </c>
       <c r="S83" s="2">
-        <v>3.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="84" spans="1:19">
@@ -13720,10 +13720,10 @@
         <v>324792</v>
       </c>
       <c r="Q84" s="1">
-        <v>3552</v>
+        <v>3534</v>
       </c>
       <c r="R84" s="1">
-        <v>251520</v>
+        <v>249542</v>
       </c>
       <c r="S84" s="2">
         <v>4.4</v>
@@ -13779,10 +13779,10 @@
         <v>312069</v>
       </c>
       <c r="Q85" s="1">
-        <v>1887</v>
+        <v>1805</v>
       </c>
       <c r="R85" s="1">
-        <v>115063</v>
+        <v>112586</v>
       </c>
       <c r="S85" s="2">
         <v>1</v>
@@ -13838,10 +13838,10 @@
         <v>306511</v>
       </c>
       <c r="Q86" s="1">
-        <v>887</v>
+        <v>852</v>
       </c>
       <c r="R86" s="1">
-        <v>82365</v>
+        <v>77956</v>
       </c>
       <c r="S86" s="2">
         <v>1.2</v>
@@ -13897,13 +13897,13 @@
         <v>306374</v>
       </c>
       <c r="Q87" s="1">
-        <v>956</v>
+        <v>927</v>
       </c>
       <c r="R87" s="1">
-        <v>95158</v>
+        <v>92476</v>
       </c>
       <c r="S87" s="2">
-        <v>2</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="88" spans="1:19">
@@ -13956,10 +13956,10 @@
         <v>303328</v>
       </c>
       <c r="Q88" s="1">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="R88" s="1">
-        <v>6152</v>
+        <v>6000</v>
       </c>
       <c r="S88" s="2">
         <v>0.1</v>
@@ -14015,7 +14015,7 @@
         <v>287372</v>
       </c>
       <c r="Q89" s="1">
-        <v>1314</v>
+        <v>1324</v>
       </c>
       <c r="R89" s="1">
         <v>182207</v>
@@ -14074,10 +14074,10 @@
         <v>279120</v>
       </c>
       <c r="Q90" s="1">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="R90" s="1">
-        <v>7441</v>
+        <v>7126</v>
       </c>
       <c r="S90" s="2">
         <v>0.2</v>
@@ -14133,13 +14133,13 @@
         <v>258797</v>
       </c>
       <c r="Q91" s="1">
-        <v>871</v>
+        <v>751</v>
       </c>
       <c r="R91" s="1">
-        <v>62770</v>
+        <v>53938</v>
       </c>
       <c r="S91" s="2">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="92" spans="1:19">
@@ -14192,13 +14192,13 @@
         <v>257112</v>
       </c>
       <c r="Q92" s="1">
-        <v>623</v>
+        <v>374</v>
       </c>
       <c r="R92" s="1">
-        <v>98854</v>
+        <v>69212</v>
       </c>
       <c r="S92" s="2">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="93" spans="1:19">
@@ -14251,10 +14251,10 @@
         <v>247853</v>
       </c>
       <c r="Q93" s="1">
-        <v>5680</v>
+        <v>5678</v>
       </c>
       <c r="R93" s="1">
-        <v>824972</v>
+        <v>824852</v>
       </c>
       <c r="S93" s="2">
         <v>11.4</v>
@@ -14310,13 +14310,13 @@
         <v>247507</v>
       </c>
       <c r="Q94" s="1">
-        <v>603</v>
+        <v>610</v>
       </c>
       <c r="R94" s="1">
-        <v>102296</v>
+        <v>101210</v>
       </c>
       <c r="S94" s="2">
-        <v>1.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="95" spans="1:19">
@@ -14369,13 +14369,13 @@
         <v>232232</v>
       </c>
       <c r="Q95" s="1">
-        <v>91</v>
+        <v>34</v>
       </c>
       <c r="R95" s="1">
-        <v>18737</v>
+        <v>9155</v>
       </c>
       <c r="S95" s="2">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="96" spans="1:19">
@@ -14428,13 +14428,13 @@
         <v>228869</v>
       </c>
       <c r="Q96" s="1">
-        <v>959</v>
+        <v>834</v>
       </c>
       <c r="R96" s="1">
-        <v>61533</v>
+        <v>53338</v>
       </c>
       <c r="S96" s="2">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:19">
@@ -14487,13 +14487,13 @@
         <v>222516</v>
       </c>
       <c r="Q97" s="1">
-        <v>4873</v>
+        <v>4748</v>
       </c>
       <c r="R97" s="1">
-        <v>582922</v>
+        <v>565737</v>
       </c>
       <c r="S97" s="2">
-        <v>12</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="98" spans="1:19">
@@ -14546,10 +14546,10 @@
         <v>209820</v>
       </c>
       <c r="Q98" s="1">
-        <v>3500</v>
+        <v>3478</v>
       </c>
       <c r="R98" s="1">
-        <v>189934</v>
+        <v>188378</v>
       </c>
       <c r="S98" s="2">
         <v>5.7</v>
@@ -14605,10 +14605,10 @@
         <v>205272</v>
       </c>
       <c r="Q99" s="1">
-        <v>542</v>
+        <v>538</v>
       </c>
       <c r="R99" s="1">
-        <v>123683</v>
+        <v>122694</v>
       </c>
       <c r="S99" s="2">
         <v>2.7</v>
@@ -14664,13 +14664,13 @@
         <v>192351</v>
       </c>
       <c r="Q100" s="1">
-        <v>1500</v>
+        <v>1439</v>
       </c>
       <c r="R100" s="1">
-        <v>339352</v>
+        <v>320059</v>
       </c>
       <c r="S100" s="2">
-        <v>11.4</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="101" spans="1:19">
@@ -14723,10 +14723,10 @@
         <v>188616</v>
       </c>
       <c r="Q101" s="1">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="R101" s="1">
-        <v>58593</v>
+        <v>58343</v>
       </c>
       <c r="S101" s="2">
         <v>1.8</v>
@@ -14782,13 +14782,13 @@
         <v>181446</v>
       </c>
       <c r="Q102" s="1">
-        <v>1816</v>
+        <v>1773</v>
       </c>
       <c r="R102" s="1">
-        <v>117499</v>
+        <v>112606</v>
       </c>
       <c r="S102" s="2">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="103" spans="1:19">
@@ -14900,13 +14900,13 @@
         <v>166081</v>
       </c>
       <c r="Q104" s="1">
-        <v>1301</v>
+        <v>1273</v>
       </c>
       <c r="R104" s="1">
-        <v>115680</v>
+        <v>111075</v>
       </c>
       <c r="S104" s="2">
-        <v>2.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="105" spans="1:19">
@@ -14959,10 +14959,10 @@
         <v>165708</v>
       </c>
       <c r="Q105" s="1">
-        <v>526</v>
+        <v>505</v>
       </c>
       <c r="R105" s="1">
-        <v>26563</v>
+        <v>25766</v>
       </c>
       <c r="S105" s="2">
         <v>0.9</v>
@@ -15018,13 +15018,13 @@
         <v>162658</v>
       </c>
       <c r="Q106" s="1">
-        <v>2785</v>
+        <v>2464</v>
       </c>
       <c r="R106" s="1">
-        <v>84261</v>
+        <v>78163</v>
       </c>
       <c r="S106" s="2">
-        <v>3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="107" spans="1:19">
@@ -15077,10 +15077,10 @@
         <v>160758</v>
       </c>
       <c r="Q107" s="1">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="R107" s="1">
-        <v>119460</v>
+        <v>119198</v>
       </c>
       <c r="S107" s="2">
         <v>4.4</v>
@@ -15136,13 +15136,13 @@
         <v>155919</v>
       </c>
       <c r="Q108" s="1">
-        <v>1332</v>
+        <v>1234</v>
       </c>
       <c r="R108" s="1">
-        <v>56555</v>
+        <v>52432</v>
       </c>
       <c r="S108" s="2">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="109" spans="1:19">
@@ -15195,10 +15195,10 @@
         <v>145054</v>
       </c>
       <c r="Q109" s="1">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="R109" s="1">
-        <v>120437</v>
+        <v>118606</v>
       </c>
       <c r="S109" s="2">
         <v>3.3</v>
@@ -15254,10 +15254,10 @@
         <v>125380</v>
       </c>
       <c r="Q110" s="1">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="R110" s="1">
-        <v>37981</v>
+        <v>36241</v>
       </c>
       <c r="S110" s="2">
         <v>1.7</v>
@@ -15313,10 +15313,10 @@
         <v>119439</v>
       </c>
       <c r="Q111" s="1">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="R111" s="1">
-        <v>36824</v>
+        <v>36775</v>
       </c>
       <c r="S111" s="2">
         <v>1.8</v>
@@ -15431,13 +15431,13 @@
         <v>108899</v>
       </c>
       <c r="Q113" s="1">
-        <v>462</v>
+        <v>416</v>
       </c>
       <c r="R113" s="1">
-        <v>23593</v>
+        <v>21236</v>
       </c>
       <c r="S113" s="2">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="114" spans="1:19">
@@ -15490,13 +15490,13 @@
         <v>85756</v>
       </c>
       <c r="Q114" s="1">
-        <v>192</v>
+        <v>79</v>
       </c>
       <c r="R114" s="1">
-        <v>17455</v>
+        <v>5286</v>
       </c>
       <c r="S114" s="2">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="115" spans="1:19">
@@ -15549,10 +15549,10 @@
         <v>77595</v>
       </c>
       <c r="Q115" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R115" s="1">
-        <v>295</v>
+        <v>258</v>
       </c>
       <c r="S115" s="2">
         <v>0</v>
@@ -15667,10 +15667,10 @@
         <v>70476</v>
       </c>
       <c r="Q117" s="1">
-        <v>442</v>
+        <v>422</v>
       </c>
       <c r="R117" s="1">
-        <v>13614</v>
+        <v>13014</v>
       </c>
       <c r="S117" s="2">
         <v>1.1</v>
@@ -15726,13 +15726,13 @@
         <v>65173</v>
       </c>
       <c r="Q118" s="1">
-        <v>387</v>
+        <v>261</v>
       </c>
       <c r="R118" s="1">
-        <v>26053</v>
+        <v>19109</v>
       </c>
       <c r="S118" s="2">
-        <v>1.6</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="119" spans="1:19">
@@ -15785,13 +15785,13 @@
         <v>61440</v>
       </c>
       <c r="Q119" s="1">
-        <v>258</v>
+        <v>166</v>
       </c>
       <c r="R119" s="1">
-        <v>10610</v>
+        <v>7950</v>
       </c>
       <c r="S119" s="2">
-        <v>1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="120" spans="1:19">
@@ -15962,13 +15962,13 @@
         <v>36954</v>
       </c>
       <c r="Q122" s="1">
-        <v>2263</v>
+        <v>2186</v>
       </c>
       <c r="R122" s="1">
-        <v>67176</v>
+        <v>64866</v>
       </c>
       <c r="S122" s="2">
-        <v>11</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="123" spans="1:19">
@@ -16021,13 +16021,13 @@
         <v>34286</v>
       </c>
       <c r="Q123" s="1">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="R123" s="1">
-        <v>33886</v>
+        <v>33271</v>
       </c>
       <c r="S123" s="2">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="124" spans="1:19">
@@ -16080,10 +16080,10 @@
         <v>30897</v>
       </c>
       <c r="Q124" s="1">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="R124" s="1">
-        <v>10473</v>
+        <v>10353</v>
       </c>
       <c r="S124" s="2">
         <v>0</v>
@@ -16139,10 +16139,10 @@
         <v>25268</v>
       </c>
       <c r="Q125" s="1">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="R125" s="1">
-        <v>9855</v>
+        <v>9791</v>
       </c>
       <c r="S125" s="2">
         <v>2.5</v>
@@ -16257,13 +16257,13 @@
         <v>2439</v>
       </c>
       <c r="Q127" s="1">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="R127" s="1">
-        <v>2089</v>
+        <v>1347</v>
       </c>
       <c r="S127" s="2">
-        <v>4.8</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="128" spans="1:19">
@@ -16375,13 +16375,13 @@
         <v>94</v>
       </c>
       <c r="Q129" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="R129" s="1">
-        <v>1201</v>
+        <v>1030</v>
       </c>
       <c r="S129" s="2">
-        <v>84</v>
+        <v>72</v>
       </c>
     </row>
     <row r="130" spans="1:19">
@@ -16434,10 +16434,10 @@
         <v>0</v>
       </c>
       <c r="Q130" s="1">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="R130" s="1">
-        <v>1159</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="131" spans="1:19">
@@ -16546,10 +16546,10 @@
         <v>0</v>
       </c>
       <c r="Q132" s="1">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R132" s="1">
-        <v>556</v>
+        <v>40</v>
       </c>
     </row>
     <row r="133" spans="1:19">

</xml_diff>